<commit_message>
fix(data): Complete excluded papers list with 9 missing studies
Missing studies identified:

V5 처리 중 제외 (5개 - 원본 코딩에 있었음):
- Study 10: Etkin et al. (2025) - GPT comprehension
- Study 17: Wang & Zhang (2025) - AI writing development
- Study 20: Dai et al. (2025) - AI feedback physics
- Study 51: Banihashem et al. (2024) - AI feedback essay
- Study 56: Leong et al. (2024) - Context personalization

미코딩 (4개 - 원본에도 없음):
- Study 9, 18, 39, 61

Action required: PDF 재검토 및 데이터 복구

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/03_final/GenAI_MetaAnalysis_v5_VERIFICATION.xlsx
+++ b/data/03_final/GenAI_MetaAnalysis_v5_VERIFICATION.xlsx
@@ -38205,90 +38205,350 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Study_Info</t>
+          <t>Study_ID</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Authors</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Original_Effects</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Exclusion_Category</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>Exclusion_Reason</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>DOI</t>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Action_Required</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Study 10</t>
-        </is>
+      <c r="A2" t="n">
+        <v>10</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Not in v5 final dataset</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>Differential Effects of GPT-Based Tools on Comprehension of Standardized Passages</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Hudson K. Etkin; Kai J. Etkin; Ryan J. Carter; Camarin E. Rolle</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>V5 처리 중 제외</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>V5 데이터 처리 과정에서 누락됨 - 확인 필요</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>PDF 재검토 및 데이터 복구</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Study 17</t>
-        </is>
+      <c r="A3" t="n">
+        <v>17</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Not in v5 final dataset</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>Exploring the Role of AI Technology in Shaping College Students’ English Writing Development: Insights from the Complex Dynamic Systems Theory</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Wang Jian; Xiaohong Zhang</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>V5 처리 중 제외</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>V5 데이터 처리 과정에서 누락됨 - 확인 필요</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PDF 재검토 및 데이터 복구</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Study 51</t>
-        </is>
+      <c r="A4" t="n">
+        <v>20</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Not in v5 final dataset</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>How Students Use AI Feedback Matters: Experimental Evidence on Physics Achievement and Autonomy</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Xusheng Dai; Zhaochun Wen; Jianxiao Jiang; Huiqin Liu; Yu Zhang</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>V5 처리 중 제외</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>V5 데이터 처리 과정에서 누락됨 - 확인 필요</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>PDF 재검토 및 데이터 복구</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Study 20</t>
-        </is>
+      <c r="A5" t="n">
+        <v>51</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Not in v5 final dataset</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>Feedback sources in essay writing: peer-generated or AI-generated feedback?</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Seyyed Kazem Banihashem; Nafiseh Taghizadeh Kerman; Omid Noroozi; Jewoong Moon; Hendrik Drachsler</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>V5 처리 중 제외</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>V5 데이터 처리 과정에서 누락됨 - 확인 필요</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>PDF 재검토 및 데이터 복구</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Study 56</t>
-        </is>
+      <c r="A6" t="n">
+        <v>56</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Not in v5 final dataset</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>Putting Things into Context: Generative AI-Enabled Context Personalization for Vocabulary Learning Improves Learning Motivation</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Joanne Leong; Pat Pataranutaporn; Valdemar Danry; Florian Perteneder; Yaoli Mao; Pattie Maes</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>V5 처리 중 제외</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>V5 데이터 처리 과정에서 누락됨 - 확인 필요</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>PDF 재검토 및 데이터 복구</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Not coded</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>미코딩</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>원본 코딩 데이터에 포함되지 않음</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>PDF 확인 - 포함 기준 충족 여부 검토</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>18</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Not coded</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>미코딩</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>원본 코딩 데이터에 포함되지 않음</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>PDF 확인 - 포함 기준 충족 여부 검토</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>39</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Not coded</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>미코딩</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>원본 코딩 데이터에 포함되지 않음</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>PDF 확인 - 포함 기준 충족 여부 검토</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>61</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Not coded</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>미코딩</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>원본 코딩 데이터에 포함되지 않음</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>PDF 확인 - 포함 기준 충족 여부 검토</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -38301,7 +38561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38317,14 +38577,14 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Percentage</t>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>총 연구 수</t>
+          <t>총 연구 수 (V5)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -38332,7 +38592,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>1-70 범위 중 61개</t>
         </is>
       </c>
     </row>
@@ -38345,11 +38605,7 @@
       <c r="B3" t="n">
         <v>346</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -38360,11 +38616,7 @@
       <c r="B4" t="n">
         <v>164</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>47.4%</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -38375,11 +38627,7 @@
       <c r="B5" t="n">
         <v>196</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>56.6%</t>
-        </is>
-      </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -38390,11 +38638,7 @@
       <c r="B6" t="n">
         <v>182</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>52.6%</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -38405,11 +38649,7 @@
       <c r="B7" t="n">
         <v>167</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>24.1%</t>
-        </is>
-      </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -38420,11 +38660,7 @@
       <c r="B8" t="n">
         <v>295</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>42.6%</t>
-        </is>
-      </c>
+      <c r="C8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -38435,24 +38671,50 @@
       <c r="B9" t="n">
         <v>131</v>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>18.9%</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>제외 논문 수</t>
+          <t>제외/누락 논문 수</t>
         </is>
       </c>
       <c r="B10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Study IDs: [9, np.int64(10), np.int64(17), 18, np.int64(20), 39, np.int64(51), np.int64(56), 61]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>- V5 처리 중 제외</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>5</v>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>IDs: [np.int64(10), np.int64(17), np.int64(20), np.int64(51), np.int64(56)]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>- 미코딩</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>IDs: [9, 18, 39, 61]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add Study 70 PDF and clarify uncoded papers status
Added:
- pdfs/070_Yilmaz_2023_Effect_of_Generative_AI_on_Computational_Thinking.pdf

Clarified 4 uncoded papers (NOT excluded, status undetermined):
- Study 9: Rommel (2025) - Adaptive and emotionally responsive
- Study 18: Satoru (2025) - CEFR Levels Evaluating
- Study 39: Jenny (2025) - Psychological topic
- Study 61: Pablo (2024) - Scientific Information thinking

These papers have PDFs but were never coded.
Action required: Full-text review to determine inclusion/exclusion.

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/03_final/GenAI_MetaAnalysis_v5_VERIFICATION.xlsx
+++ b/data/03_final/GenAI_MetaAnalysis_v5_VERIFICATION.xlsx
@@ -10,7 +10,7 @@
     <sheet name="1_Codebook" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="2_Effect_Sizes_Verification" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3_Study_Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4_Excluded_Papers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="4_Uncoded_Papers" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5_Statistics" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
@@ -35599,7 +35599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35610,22 +35610,27 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>PDF_File</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Exclusion_Category</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Exclusion_Reason</t>
+          <t>Possible_Reason</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
           <t>Action_Required</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
@@ -35635,22 +35640,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Not coded</t>
+          <t>009_Rommel_2025_Development_of_adaptive_and_emotionally_.pdf</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>미코딩</t>
+          <t>PDF 있음, 미코딩</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>PDF는 있으나 코딩되지 않음</t>
+          <t>검토 필요 - 포함/제외 결정 미정</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>PDF 검토 필요</t>
+          <t>PDF 전문 검토 후 포함/제외 결정</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Rommel (2025) - Adaptive and emotionally responsive</t>
         </is>
       </c>
     </row>
@@ -35660,22 +35670,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Not coded</t>
+          <t>018_Satoru_2025_Generative_AI_and_CEFR_Levels_Evaluating.pdf</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>미코딩</t>
+          <t>PDF 있음, 미코딩</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>PDF는 있으나 코딩되지 않음</t>
+          <t>검토 필요 - 포함/제외 결정 미정</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PDF 검토 필요</t>
+          <t>PDF 전문 검토 후 포함/제외 결정</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Satoru (2025) - CEFR Levels Evaluating</t>
         </is>
       </c>
     </row>
@@ -35685,22 +35700,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Not coded</t>
+          <t>039_Jenny_2025_Using_Generative_AI_to_Promote_Psycholog.pdf</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>미코딩</t>
+          <t>PDF 있음, 미코딩</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PDF는 있으나 코딩되지 않음</t>
+          <t>검토 필요 - 포함/제외 결정 미정</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PDF 검토 필요</t>
+          <t>PDF 전문 검토 후 포함/제외 결정</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Jenny (2025) - Psychological topic</t>
         </is>
       </c>
     </row>
@@ -35710,22 +35730,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Not coded</t>
+          <t>061_Pablo_2024_Thinking_Critically_about_Scientific_Inf.pdf</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>미코딩</t>
+          <t>PDF 있음, 미코딩</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PDF는 있으나 코딩되지 않음</t>
+          <t>검토 필요 - 포함/제외 결정 미정</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PDF 검토 필요</t>
+          <t>PDF 전문 검토 후 포함/제외 결정</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pablo (2024) - Scientific Information thinking</t>
         </is>
       </c>
     </row>
@@ -35740,7 +35765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35763,7 +35788,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>총 연구 수</t>
+          <t>총 연구 수 (V5)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -35771,7 +35796,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>66개 (5개 복구됨)</t>
+          <t>Study 1-70 중 66개</t>
         </is>
       </c>
     </row>
@@ -35786,52 +35811,67 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>375개 (29개 복구됨)</t>
+          <t>5개 연구 복구 포함</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hedges_g 있음</t>
+          <t>복구된 연구</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>217</v>
+        <v>5</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>57.9%</t>
+          <t>Study 10, 17, 20, 51, 56</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>검토 필요</t>
+          <t>Hedges_g 있음</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>198</v>
+        <v>217</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>57.9%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>미코딩 연구</t>
+          <t>검토 필요</t>
         </is>
       </c>
       <c r="B6" t="n">
+        <v>198</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>198/375</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PDF 있으나 미코딩 (상태 미정)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>4</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Study 9, 18, 39, 61</t>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Study 9, 18, 39, 61 - 포함/제외 결정 필요</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Update excluded papers list and regenerate PDF_INDEX.md
- Add 4 excluded studies (9, 18, 39, 61) with exclusion reasons to VERIFICATION.xlsx
- Regenerate PDF_INDEX.md with 66 included, 4 excluded studies
- Total: 70 PDFs, 375 effect sizes in V5
- Add automation script update_excluded_and_index.py for future updates

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/03_final/GenAI_MetaAnalysis_v5_VERIFICATION.xlsx
+++ b/data/03_final/GenAI_MetaAnalysis_v5_VERIFICATION.xlsx
@@ -12,6 +12,7 @@
     <sheet name="3_Study_Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4_Uncoded_Papers" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5_Statistics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5_Excluded_Papers" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,8 +454,6 @@
           <t>연구 고유 ID</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -467,8 +466,6 @@
           <t>효과크기 ID</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -481,8 +478,6 @@
           <t>논문 제목</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -495,8 +490,6 @@
           <t>출판 연도</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -509,8 +502,6 @@
           <t>저자</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -523,8 +514,6 @@
           <t>결과변수 이름</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -537,8 +526,6 @@
           <t>결과 차원</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -551,8 +538,6 @@
           <t>Bloom 분류</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -565,8 +550,6 @@
           <t>처치군 n</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -579,8 +562,6 @@
           <t>통제군 n</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -593,8 +574,6 @@
           <t>처치군 평균</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -607,8 +586,6 @@
           <t>처치군 SD</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -621,8 +598,6 @@
           <t>통제군 평균</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -635,8 +610,6 @@
           <t>통제군 SD</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -649,8 +622,6 @@
           <t>Hedges g</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -663,8 +634,6 @@
           <t>SE</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -677,8 +646,6 @@
           <t>검증 상태</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -691,8 +658,6 @@
           <t>검증 신뢰도</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -705,8 +670,6 @@
           <t>데이터 등급</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -719,8 +682,6 @@
           <t>AI 도구</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -733,8 +694,6 @@
           <t>연구 설계</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -909,7 +868,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -998,7 +956,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -1087,7 +1044,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -1176,7 +1132,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -1358,7 +1313,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -1378,13 +1332,9 @@
       <c r="O7" t="n">
         <v>3.63</v>
       </c>
-      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
         <v>3.19</v>
       </c>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -1439,7 +1389,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -1459,13 +1408,9 @@
       <c r="O8" t="n">
         <v>3.54</v>
       </c>
-      <c r="P8" t="inlineStr"/>
       <c r="Q8" t="n">
         <v>3.22</v>
       </c>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -1505,7 +1450,6 @@
       <c r="F9" t="n">
         <v>2025</v>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Academic Writing Achievement Pre-Test</t>
@@ -1594,7 +1538,6 @@
       <c r="F10" t="n">
         <v>2025</v>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Academic Writing Achievement Post-Test</t>
@@ -1698,7 +1641,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -1787,7 +1729,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -1876,7 +1817,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -1965,7 +1905,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -2426,7 +2365,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -2515,7 +2453,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -3012,7 +2949,6 @@
       <c r="S25" t="n">
         <v>1.3059</v>
       </c>
-      <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -3103,7 +3039,6 @@
       <c r="S26" t="n">
         <v>1.1962</v>
       </c>
-      <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -3194,7 +3129,6 @@
       <c r="S27" t="n">
         <v>1.1165</v>
       </c>
-      <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -3285,7 +3219,6 @@
       <c r="S28" t="n">
         <v>0.9669</v>
       </c>
-      <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -3376,7 +3309,6 @@
       <c r="S29" t="n">
         <v>0.8772</v>
       </c>
-      <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -3467,7 +3399,6 @@
       <c r="S30" t="n">
         <v>1.266</v>
       </c>
-      <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -3522,7 +3453,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
       <c r="K31" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -3539,12 +3469,6 @@
       <c r="N31" t="n">
         <v>120</v>
       </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
-      <c r="S31" t="inlineStr"/>
-      <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -3589,9 +3513,6 @@
           <t>Wesley Wu-Yi Koo</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
       <c r="K32" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -3602,14 +3523,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
-      <c r="S32" t="inlineStr"/>
-      <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -4036,7 +3949,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -4422,15 +4334,9 @@
       <c r="M41" t="n">
         <v>70</v>
       </c>
-      <c r="N41" t="inlineStr"/>
       <c r="O41" t="n">
         <v>2.2</v>
       </c>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-      <c r="S41" t="inlineStr"/>
-      <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -4503,15 +4409,9 @@
       <c r="M42" t="n">
         <v>52</v>
       </c>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" t="n">
         <v>2.5</v>
       </c>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
-      <c r="S42" t="inlineStr"/>
-      <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -4584,15 +4484,9 @@
       <c r="M43" t="n">
         <v>70</v>
       </c>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" t="n">
         <v>2.9</v>
       </c>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
-      <c r="S43" t="inlineStr"/>
-      <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -4632,7 +4526,6 @@
       <c r="F44" t="n">
         <v>2025</v>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>theoretical knowledge test</t>
@@ -4664,14 +4557,9 @@
       <c r="N44" t="n">
         <v>20</v>
       </c>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
-      <c r="Q44" t="inlineStr"/>
-      <c r="R44" t="inlineStr"/>
       <c r="S44" t="n">
         <v>3.0776</v>
       </c>
-      <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -4711,7 +4599,6 @@
       <c r="F45" t="n">
         <v>2025</v>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>Mini Clinical Evaluation Exercise</t>
@@ -4743,12 +4630,6 @@
       <c r="N45" t="n">
         <v>20</v>
       </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
-      <c r="S45" t="inlineStr"/>
-      <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -4788,7 +4669,6 @@
       <c r="F46" t="n">
         <v>2025</v>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>AI self-efficacy</t>
@@ -4799,7 +4679,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -4816,14 +4695,9 @@
       <c r="N46" t="n">
         <v>20</v>
       </c>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
-      <c r="Q46" t="inlineStr"/>
-      <c r="R46" t="inlineStr"/>
       <c r="S46" t="n">
         <v>1.6662</v>
       </c>
-      <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -4863,7 +4737,6 @@
       <c r="F47" t="n">
         <v>2025</v>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>internet addiction</t>
@@ -4874,7 +4747,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -4891,12 +4763,6 @@
       <c r="N47" t="n">
         <v>20</v>
       </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
-      <c r="Q47" t="inlineStr"/>
-      <c r="R47" t="inlineStr"/>
-      <c r="S47" t="inlineStr"/>
-      <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -4936,7 +4802,6 @@
       <c r="F48" t="n">
         <v>2025</v>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>reading motivation</t>
@@ -4947,7 +4812,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -4964,14 +4828,9 @@
       <c r="N48" t="n">
         <v>20</v>
       </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
-      <c r="Q48" t="inlineStr"/>
-      <c r="R48" t="inlineStr"/>
       <c r="S48" t="n">
         <v>1.284</v>
       </c>
-      <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5047,12 +4906,6 @@
       <c r="N49" t="n">
         <v>134</v>
       </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
-      <c r="R49" t="inlineStr"/>
-      <c r="S49" t="inlineStr"/>
-      <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5128,12 +4981,6 @@
       <c r="N50" t="n">
         <v>134</v>
       </c>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
-      <c r="Q50" t="inlineStr"/>
-      <c r="R50" t="inlineStr"/>
-      <c r="S50" t="inlineStr"/>
-      <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5209,12 +5056,6 @@
       <c r="N51" t="n">
         <v>134</v>
       </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="inlineStr"/>
-      <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5290,12 +5131,6 @@
       <c r="N52" t="n">
         <v>134</v>
       </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
-      <c r="Q52" t="inlineStr"/>
-      <c r="R52" t="inlineStr"/>
-      <c r="S52" t="inlineStr"/>
-      <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5350,7 +5185,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -5367,12 +5201,6 @@
       <c r="N53" t="n">
         <v>134</v>
       </c>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
-      <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5427,7 +5255,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -5444,12 +5271,6 @@
       <c r="N54" t="n">
         <v>134</v>
       </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
       <c r="U54" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5504,7 +5325,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -5521,12 +5341,6 @@
       <c r="N55" t="n">
         <v>134</v>
       </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
-      <c r="T55" t="inlineStr"/>
       <c r="U55" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5581,7 +5395,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -5598,12 +5411,6 @@
       <c r="N56" t="n">
         <v>134</v>
       </c>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
-      <c r="T56" t="inlineStr"/>
       <c r="U56" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5658,7 +5465,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -5747,7 +5553,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -5761,13 +5566,6 @@
       <c r="M58" t="n">
         <v>125</v>
       </c>
-      <c r="N58" t="inlineStr"/>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
-      <c r="T58" t="inlineStr"/>
       <c r="U58" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -5915,7 +5713,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -6025,12 +5822,6 @@
       <c r="N61" t="n">
         <v>70</v>
       </c>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
-      <c r="T61" t="inlineStr"/>
       <c r="U61" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -6106,12 +5897,6 @@
       <c r="N62" t="n">
         <v>33</v>
       </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
-      <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -6166,7 +5951,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -6255,7 +6039,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -6344,7 +6127,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -6433,7 +6215,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -6522,7 +6303,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -6611,7 +6391,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -6700,7 +6479,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -6717,12 +6495,6 @@
       <c r="N69" t="n">
         <v>33</v>
       </c>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
-      <c r="T69" t="inlineStr"/>
       <c r="U69" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -6777,7 +6549,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -6794,12 +6565,6 @@
       <c r="N70" t="n">
         <v>33</v>
       </c>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
-      <c r="T70" t="inlineStr"/>
       <c r="U70" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -6854,7 +6619,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -6871,12 +6635,6 @@
       <c r="N71" t="n">
         <v>33</v>
       </c>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
-      <c r="T71" t="inlineStr"/>
       <c r="U71" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -6955,13 +6713,9 @@
       <c r="O72" t="n">
         <v>410.7</v>
       </c>
-      <c r="P72" t="inlineStr"/>
       <c r="Q72" t="n">
         <v>80.7</v>
       </c>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
-      <c r="T72" t="inlineStr"/>
       <c r="U72" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -7040,13 +6794,9 @@
       <c r="O73" t="n">
         <v>291</v>
       </c>
-      <c r="P73" t="inlineStr"/>
       <c r="Q73" t="n">
         <v>290.8</v>
       </c>
-      <c r="R73" t="inlineStr"/>
-      <c r="S73" t="inlineStr"/>
-      <c r="T73" t="inlineStr"/>
       <c r="U73" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -7137,7 +6887,6 @@
       <c r="S74" t="n">
         <v>0.0297</v>
       </c>
-      <c r="T74" t="inlineStr"/>
       <c r="U74" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -7228,7 +6977,6 @@
       <c r="S75" t="n">
         <v>0.2273</v>
       </c>
-      <c r="T75" t="inlineStr"/>
       <c r="U75" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -7319,7 +7067,6 @@
       <c r="S76" t="n">
         <v>0.0689</v>
       </c>
-      <c r="T76" t="inlineStr"/>
       <c r="U76" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -7410,7 +7157,6 @@
       <c r="S77" t="n">
         <v>0.71</v>
       </c>
-      <c r="T77" t="inlineStr"/>
       <c r="U77" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -7501,7 +7247,6 @@
       <c r="S78" t="n">
         <v>0.6691</v>
       </c>
-      <c r="T78" t="inlineStr"/>
       <c r="U78" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -7592,7 +7337,6 @@
       <c r="S79" t="n">
         <v>0.2169</v>
       </c>
-      <c r="T79" t="inlineStr"/>
       <c r="U79" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -7683,7 +7427,6 @@
       <c r="S80" t="n">
         <v>0.3355</v>
       </c>
-      <c r="T80" t="inlineStr"/>
       <c r="U80" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -7756,13 +7499,6 @@
       <c r="M81" t="n">
         <v>12</v>
       </c>
-      <c r="N81" t="inlineStr"/>
-      <c r="O81" t="inlineStr"/>
-      <c r="P81" t="inlineStr"/>
-      <c r="Q81" t="inlineStr"/>
-      <c r="R81" t="inlineStr"/>
-      <c r="S81" t="inlineStr"/>
-      <c r="T81" t="inlineStr"/>
       <c r="U81" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -7835,13 +7571,6 @@
       <c r="M82" t="n">
         <v>12</v>
       </c>
-      <c r="N82" t="inlineStr"/>
-      <c r="O82" t="inlineStr"/>
-      <c r="P82" t="inlineStr"/>
-      <c r="Q82" t="inlineStr"/>
-      <c r="R82" t="inlineStr"/>
-      <c r="S82" t="inlineStr"/>
-      <c r="T82" t="inlineStr"/>
       <c r="U82" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -7914,13 +7643,6 @@
       <c r="M83" t="n">
         <v>12</v>
       </c>
-      <c r="N83" t="inlineStr"/>
-      <c r="O83" t="inlineStr"/>
-      <c r="P83" t="inlineStr"/>
-      <c r="Q83" t="inlineStr"/>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="inlineStr"/>
-      <c r="T83" t="inlineStr"/>
       <c r="U83" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -7993,13 +7715,6 @@
       <c r="M84" t="n">
         <v>12</v>
       </c>
-      <c r="N84" t="inlineStr"/>
-      <c r="O84" t="inlineStr"/>
-      <c r="P84" t="inlineStr"/>
-      <c r="Q84" t="inlineStr"/>
-      <c r="R84" t="inlineStr"/>
-      <c r="S84" t="inlineStr"/>
-      <c r="T84" t="inlineStr"/>
       <c r="U84" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8072,13 +7787,6 @@
       <c r="M85" t="n">
         <v>12</v>
       </c>
-      <c r="N85" t="inlineStr"/>
-      <c r="O85" t="inlineStr"/>
-      <c r="P85" t="inlineStr"/>
-      <c r="Q85" t="inlineStr"/>
-      <c r="R85" t="inlineStr"/>
-      <c r="S85" t="inlineStr"/>
-      <c r="T85" t="inlineStr"/>
       <c r="U85" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8340,14 +8048,9 @@
       <c r="N88" t="n">
         <v>38</v>
       </c>
-      <c r="O88" t="inlineStr"/>
-      <c r="P88" t="inlineStr"/>
-      <c r="Q88" t="inlineStr"/>
-      <c r="R88" t="inlineStr"/>
       <c r="S88" t="n">
         <v>0.6665</v>
       </c>
-      <c r="T88" t="inlineStr"/>
       <c r="U88" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8423,14 +8126,9 @@
       <c r="N89" t="n">
         <v>38</v>
       </c>
-      <c r="O89" t="inlineStr"/>
-      <c r="P89" t="inlineStr"/>
-      <c r="Q89" t="inlineStr"/>
-      <c r="R89" t="inlineStr"/>
       <c r="S89" t="n">
         <v>-0.5338000000000001</v>
       </c>
-      <c r="T89" t="inlineStr"/>
       <c r="U89" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8506,14 +8204,9 @@
       <c r="N90" t="n">
         <v>38</v>
       </c>
-      <c r="O90" t="inlineStr"/>
-      <c r="P90" t="inlineStr"/>
-      <c r="Q90" t="inlineStr"/>
-      <c r="R90" t="inlineStr"/>
       <c r="S90" t="n">
         <v>-0.4724</v>
       </c>
-      <c r="T90" t="inlineStr"/>
       <c r="U90" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8589,14 +8282,9 @@
       <c r="N91" t="n">
         <v>88</v>
       </c>
-      <c r="O91" t="inlineStr"/>
-      <c r="P91" t="inlineStr"/>
-      <c r="Q91" t="inlineStr"/>
-      <c r="R91" t="inlineStr"/>
       <c r="S91" t="n">
         <v>0.3764</v>
       </c>
-      <c r="T91" t="inlineStr"/>
       <c r="U91" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8672,14 +8360,9 @@
       <c r="N92" t="n">
         <v>88</v>
       </c>
-      <c r="O92" t="inlineStr"/>
-      <c r="P92" t="inlineStr"/>
-      <c r="Q92" t="inlineStr"/>
-      <c r="R92" t="inlineStr"/>
       <c r="S92" t="n">
         <v>-0.2728</v>
       </c>
-      <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8755,14 +8438,9 @@
       <c r="N93" t="n">
         <v>88</v>
       </c>
-      <c r="O93" t="inlineStr"/>
-      <c r="P93" t="inlineStr"/>
-      <c r="Q93" t="inlineStr"/>
-      <c r="R93" t="inlineStr"/>
       <c r="S93" t="n">
         <v>-0.3913</v>
       </c>
-      <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8838,14 +8516,9 @@
       <c r="N94" t="n">
         <v>88</v>
       </c>
-      <c r="O94" t="inlineStr"/>
-      <c r="P94" t="inlineStr"/>
-      <c r="Q94" t="inlineStr"/>
-      <c r="R94" t="inlineStr"/>
       <c r="S94" t="n">
         <v>-0.2977</v>
       </c>
-      <c r="T94" t="inlineStr"/>
       <c r="U94" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -8921,14 +8594,9 @@
       <c r="N95" t="n">
         <v>88</v>
       </c>
-      <c r="O95" t="inlineStr"/>
-      <c r="P95" t="inlineStr"/>
-      <c r="Q95" t="inlineStr"/>
-      <c r="R95" t="inlineStr"/>
       <c r="S95" t="n">
         <v>-0.5466</v>
       </c>
-      <c r="T95" t="inlineStr"/>
       <c r="U95" t="inlineStr">
         <is>
           <t>RECOVERED</t>
@@ -9355,7 +9023,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -9444,7 +9111,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -9533,7 +9199,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -10180,7 +9845,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr"/>
       <c r="K109" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -10197,12 +9861,6 @@
       <c r="N109" t="n">
         <v>15</v>
       </c>
-      <c r="O109" t="inlineStr"/>
-      <c r="P109" t="inlineStr"/>
-      <c r="Q109" t="inlineStr"/>
-      <c r="R109" t="inlineStr"/>
-      <c r="S109" t="inlineStr"/>
-      <c r="T109" t="inlineStr"/>
       <c r="U109" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -10272,8 +9930,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr"/>
-      <c r="N110" t="inlineStr"/>
       <c r="O110" t="n">
         <v>12.6</v>
       </c>
@@ -10286,8 +9942,6 @@
       <c r="R110" t="n">
         <v>12.7</v>
       </c>
-      <c r="S110" t="inlineStr"/>
-      <c r="T110" t="inlineStr"/>
       <c r="U110" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10357,8 +10011,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr"/>
-      <c r="N111" t="inlineStr"/>
       <c r="O111" t="n">
         <v>13.6</v>
       </c>
@@ -10371,8 +10023,6 @@
       <c r="R111" t="n">
         <v>12</v>
       </c>
-      <c r="S111" t="inlineStr"/>
-      <c r="T111" t="inlineStr"/>
       <c r="U111" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10442,8 +10092,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M112" t="inlineStr"/>
-      <c r="N112" t="inlineStr"/>
       <c r="O112" t="n">
         <v>11.6</v>
       </c>
@@ -10456,8 +10104,6 @@
       <c r="R112" t="n">
         <v>13.5</v>
       </c>
-      <c r="S112" t="inlineStr"/>
-      <c r="T112" t="inlineStr"/>
       <c r="U112" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10527,8 +10173,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M113" t="inlineStr"/>
-      <c r="N113" t="inlineStr"/>
       <c r="O113" t="n">
         <v>16.9</v>
       </c>
@@ -10541,8 +10185,6 @@
       <c r="R113" t="n">
         <v>6.3</v>
       </c>
-      <c r="S113" t="inlineStr"/>
-      <c r="T113" t="inlineStr"/>
       <c r="U113" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10612,8 +10254,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M114" t="inlineStr"/>
-      <c r="N114" t="inlineStr"/>
       <c r="O114" t="n">
         <v>15.6</v>
       </c>
@@ -10626,8 +10266,6 @@
       <c r="R114" t="n">
         <v>13.7</v>
       </c>
-      <c r="S114" t="inlineStr"/>
-      <c r="T114" t="inlineStr"/>
       <c r="U114" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10697,8 +10335,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M115" t="inlineStr"/>
-      <c r="N115" t="inlineStr"/>
       <c r="O115" t="n">
         <v>10.7</v>
       </c>
@@ -10711,8 +10347,6 @@
       <c r="R115" t="n">
         <v>11.3</v>
       </c>
-      <c r="S115" t="inlineStr"/>
-      <c r="T115" t="inlineStr"/>
       <c r="U115" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10782,8 +10416,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M116" t="inlineStr"/>
-      <c r="N116" t="inlineStr"/>
       <c r="O116" t="n">
         <v>11.2</v>
       </c>
@@ -10796,8 +10428,6 @@
       <c r="R116" t="n">
         <v>11.2</v>
       </c>
-      <c r="S116" t="inlineStr"/>
-      <c r="T116" t="inlineStr"/>
       <c r="U116" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10867,8 +10497,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M117" t="inlineStr"/>
-      <c r="N117" t="inlineStr"/>
       <c r="O117" t="n">
         <v>7.5</v>
       </c>
@@ -10881,8 +10509,6 @@
       <c r="R117" t="n">
         <v>13.6</v>
       </c>
-      <c r="S117" t="inlineStr"/>
-      <c r="T117" t="inlineStr"/>
       <c r="U117" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -10952,8 +10578,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M118" t="inlineStr"/>
-      <c r="N118" t="inlineStr"/>
       <c r="O118" t="n">
         <v>9.199999999999999</v>
       </c>
@@ -10966,8 +10590,6 @@
       <c r="R118" t="n">
         <v>10.8</v>
       </c>
-      <c r="S118" t="inlineStr"/>
-      <c r="T118" t="inlineStr"/>
       <c r="U118" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -11037,8 +10659,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M119" t="inlineStr"/>
-      <c r="N119" t="inlineStr"/>
       <c r="O119" t="n">
         <v>10.8</v>
       </c>
@@ -11051,8 +10671,6 @@
       <c r="R119" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="S119" t="inlineStr"/>
-      <c r="T119" t="inlineStr"/>
       <c r="U119" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -11122,8 +10740,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M120" t="inlineStr"/>
-      <c r="N120" t="inlineStr"/>
       <c r="O120" t="n">
         <v>18</v>
       </c>
@@ -11136,8 +10752,6 @@
       <c r="R120" t="n">
         <v>13.3</v>
       </c>
-      <c r="S120" t="inlineStr"/>
-      <c r="T120" t="inlineStr"/>
       <c r="U120" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -11858,18 +11472,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M128" t="inlineStr"/>
-      <c r="N128" t="inlineStr"/>
       <c r="O128" t="n">
         <v>0.83</v>
       </c>
-      <c r="P128" t="inlineStr"/>
       <c r="Q128" t="n">
         <v>0.44</v>
       </c>
-      <c r="R128" t="inlineStr"/>
-      <c r="S128" t="inlineStr"/>
-      <c r="T128" t="inlineStr"/>
       <c r="U128" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -11939,18 +11547,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M129" t="inlineStr"/>
-      <c r="N129" t="inlineStr"/>
       <c r="O129" t="n">
         <v>0.95</v>
       </c>
-      <c r="P129" t="inlineStr"/>
       <c r="Q129" t="n">
         <v>0.7</v>
       </c>
-      <c r="R129" t="inlineStr"/>
-      <c r="S129" t="inlineStr"/>
-      <c r="T129" t="inlineStr"/>
       <c r="U129" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12020,18 +11622,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M130" t="inlineStr"/>
-      <c r="N130" t="inlineStr"/>
       <c r="O130" t="n">
         <v>0.62</v>
       </c>
-      <c r="P130" t="inlineStr"/>
       <c r="Q130" t="n">
         <v>0</v>
       </c>
-      <c r="R130" t="inlineStr"/>
-      <c r="S130" t="inlineStr"/>
-      <c r="T130" t="inlineStr"/>
       <c r="U130" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12101,18 +11697,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M131" t="inlineStr"/>
-      <c r="N131" t="inlineStr"/>
       <c r="O131" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="P131" t="inlineStr"/>
       <c r="Q131" t="n">
         <v>0.77</v>
       </c>
-      <c r="R131" t="inlineStr"/>
-      <c r="S131" t="inlineStr"/>
-      <c r="T131" t="inlineStr"/>
       <c r="U131" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12182,18 +11772,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M132" t="inlineStr"/>
-      <c r="N132" t="inlineStr"/>
       <c r="O132" t="n">
         <v>0.65</v>
       </c>
-      <c r="P132" t="inlineStr"/>
       <c r="Q132" t="n">
         <v>0.08</v>
       </c>
-      <c r="R132" t="inlineStr"/>
-      <c r="S132" t="inlineStr"/>
-      <c r="T132" t="inlineStr"/>
       <c r="U132" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12263,18 +11847,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M133" t="inlineStr"/>
-      <c r="N133" t="inlineStr"/>
       <c r="O133" t="n">
         <v>0.82</v>
       </c>
-      <c r="P133" t="inlineStr"/>
       <c r="Q133" t="n">
         <v>0.25</v>
       </c>
-      <c r="R133" t="inlineStr"/>
-      <c r="S133" t="inlineStr"/>
-      <c r="T133" t="inlineStr"/>
       <c r="U133" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12344,18 +11922,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M134" t="inlineStr"/>
-      <c r="N134" t="inlineStr"/>
       <c r="O134" t="n">
         <v>0.39</v>
       </c>
-      <c r="P134" t="inlineStr"/>
       <c r="Q134" t="n">
         <v>0.44</v>
       </c>
-      <c r="R134" t="inlineStr"/>
-      <c r="S134" t="inlineStr"/>
-      <c r="T134" t="inlineStr"/>
       <c r="U134" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12425,18 +11997,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M135" t="inlineStr"/>
-      <c r="N135" t="inlineStr"/>
       <c r="O135" t="n">
         <v>0.26</v>
       </c>
-      <c r="P135" t="inlineStr"/>
       <c r="Q135" t="n">
         <v>0.7</v>
       </c>
-      <c r="R135" t="inlineStr"/>
-      <c r="S135" t="inlineStr"/>
-      <c r="T135" t="inlineStr"/>
       <c r="U135" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12506,18 +12072,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M136" t="inlineStr"/>
-      <c r="N136" t="inlineStr"/>
       <c r="O136" t="n">
         <v>0.62</v>
       </c>
-      <c r="P136" t="inlineStr"/>
       <c r="Q136" t="n">
         <v>0</v>
       </c>
-      <c r="R136" t="inlineStr"/>
-      <c r="S136" t="inlineStr"/>
-      <c r="T136" t="inlineStr"/>
       <c r="U136" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12587,18 +12147,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M137" t="inlineStr"/>
-      <c r="N137" t="inlineStr"/>
       <c r="O137" t="n">
         <v>0.17</v>
       </c>
-      <c r="P137" t="inlineStr"/>
       <c r="Q137" t="n">
         <v>0.77</v>
       </c>
-      <c r="R137" t="inlineStr"/>
-      <c r="S137" t="inlineStr"/>
-      <c r="T137" t="inlineStr"/>
       <c r="U137" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12668,18 +12222,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M138" t="inlineStr"/>
-      <c r="N138" t="inlineStr"/>
       <c r="O138" t="n">
         <v>0.58</v>
       </c>
-      <c r="P138" t="inlineStr"/>
       <c r="Q138" t="n">
         <v>0.08</v>
       </c>
-      <c r="R138" t="inlineStr"/>
-      <c r="S138" t="inlineStr"/>
-      <c r="T138" t="inlineStr"/>
       <c r="U138" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -12749,18 +12297,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M139" t="inlineStr"/>
-      <c r="N139" t="inlineStr"/>
       <c r="O139" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="P139" t="inlineStr"/>
       <c r="Q139" t="n">
         <v>0.25</v>
       </c>
-      <c r="R139" t="inlineStr"/>
-      <c r="S139" t="inlineStr"/>
-      <c r="T139" t="inlineStr"/>
       <c r="U139" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -13187,7 +12729,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr"/>
       <c r="K144" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -13276,7 +12817,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr"/>
       <c r="K145" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -13365,7 +12905,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr"/>
       <c r="K146" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -13454,7 +12993,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr"/>
       <c r="K147" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -13528,7 +13066,6 @@
       <c r="F148" t="n">
         <v>2025</v>
       </c>
-      <c r="G148" t="inlineStr"/>
       <c r="H148" t="inlineStr">
         <is>
           <t>Thermodynamics Knowledge - Pretest</t>
@@ -13617,7 +13154,6 @@
       <c r="F149" t="n">
         <v>2025</v>
       </c>
-      <c r="G149" t="inlineStr"/>
       <c r="H149" t="inlineStr">
         <is>
           <t>Thermodynamics Knowledge - Posttest</t>
@@ -13664,7 +13200,6 @@
       <c r="S149" t="n">
         <v>0.6101</v>
       </c>
-      <c r="T149" t="inlineStr"/>
       <c r="U149" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -13704,7 +13239,6 @@
       <c r="F150" t="n">
         <v>2025</v>
       </c>
-      <c r="G150" t="inlineStr"/>
       <c r="H150" t="inlineStr">
         <is>
           <t>Thermodynamics Learning Gains</t>
@@ -13739,13 +13273,9 @@
       <c r="O150" t="n">
         <v>10.31</v>
       </c>
-      <c r="P150" t="inlineStr"/>
       <c r="Q150" t="n">
         <v>6.25</v>
       </c>
-      <c r="R150" t="inlineStr"/>
-      <c r="S150" t="inlineStr"/>
-      <c r="T150" t="inlineStr"/>
       <c r="U150" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -13800,7 +13330,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr"/>
       <c r="K151" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -13820,13 +13349,9 @@
       <c r="O151" t="n">
         <v>23</v>
       </c>
-      <c r="P151" t="inlineStr"/>
       <c r="Q151" t="n">
         <v>16.9</v>
       </c>
-      <c r="R151" t="inlineStr"/>
-      <c r="S151" t="inlineStr"/>
-      <c r="T151" t="inlineStr"/>
       <c r="U151" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -13881,7 +13406,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr"/>
       <c r="K152" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -13901,13 +13425,9 @@
       <c r="O152" t="n">
         <v>13.6</v>
       </c>
-      <c r="P152" t="inlineStr"/>
       <c r="Q152" t="n">
         <v>9.6</v>
       </c>
-      <c r="R152" t="inlineStr"/>
-      <c r="S152" t="inlineStr"/>
-      <c r="T152" t="inlineStr"/>
       <c r="U152" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -13962,7 +13482,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr"/>
       <c r="K153" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -13982,13 +13501,9 @@
       <c r="O153" t="n">
         <v>9.5</v>
       </c>
-      <c r="P153" t="inlineStr"/>
       <c r="Q153" t="n">
         <v>7.3</v>
       </c>
-      <c r="R153" t="inlineStr"/>
-      <c r="S153" t="inlineStr"/>
-      <c r="T153" t="inlineStr"/>
       <c r="U153" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14067,13 +13582,9 @@
       <c r="O154" t="n">
         <v>5.6</v>
       </c>
-      <c r="P154" t="inlineStr"/>
       <c r="Q154" t="n">
         <v>4.1</v>
       </c>
-      <c r="R154" t="inlineStr"/>
-      <c r="S154" t="inlineStr"/>
-      <c r="T154" t="inlineStr"/>
       <c r="U154" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14152,13 +13663,9 @@
       <c r="O155" t="n">
         <v>5.6</v>
       </c>
-      <c r="P155" t="inlineStr"/>
       <c r="Q155" t="n">
         <v>4.1</v>
       </c>
-      <c r="R155" t="inlineStr"/>
-      <c r="S155" t="inlineStr"/>
-      <c r="T155" t="inlineStr"/>
       <c r="U155" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14237,13 +13744,9 @@
       <c r="O156" t="n">
         <v>2.6</v>
       </c>
-      <c r="P156" t="inlineStr"/>
       <c r="Q156" t="n">
         <v>2.6</v>
       </c>
-      <c r="R156" t="inlineStr"/>
-      <c r="S156" t="inlineStr"/>
-      <c r="T156" t="inlineStr"/>
       <c r="U156" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14322,13 +13825,9 @@
       <c r="O157" t="n">
         <v>1.9</v>
       </c>
-      <c r="P157" t="inlineStr"/>
       <c r="Q157" t="n">
         <v>1.3</v>
       </c>
-      <c r="R157" t="inlineStr"/>
-      <c r="S157" t="inlineStr"/>
-      <c r="T157" t="inlineStr"/>
       <c r="U157" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14407,13 +13906,9 @@
       <c r="O158" t="n">
         <v>1.1</v>
       </c>
-      <c r="P158" t="inlineStr"/>
       <c r="Q158" t="n">
         <v>0.3</v>
       </c>
-      <c r="R158" t="inlineStr"/>
-      <c r="S158" t="inlineStr"/>
-      <c r="T158" t="inlineStr"/>
       <c r="U158" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14492,13 +13987,9 @@
       <c r="O159" t="n">
         <v>5.5</v>
       </c>
-      <c r="P159" t="inlineStr"/>
       <c r="Q159" t="n">
         <v>4.6</v>
       </c>
-      <c r="R159" t="inlineStr"/>
-      <c r="S159" t="inlineStr"/>
-      <c r="T159" t="inlineStr"/>
       <c r="U159" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14577,13 +14068,9 @@
       <c r="O160" t="n">
         <v>2.6</v>
       </c>
-      <c r="P160" t="inlineStr"/>
       <c r="Q160" t="n">
         <v>2.6</v>
       </c>
-      <c r="R160" t="inlineStr"/>
-      <c r="S160" t="inlineStr"/>
-      <c r="T160" t="inlineStr"/>
       <c r="U160" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14662,13 +14149,9 @@
       <c r="O161" t="n">
         <v>1.7</v>
       </c>
-      <c r="P161" t="inlineStr"/>
       <c r="Q161" t="n">
         <v>1.5</v>
       </c>
-      <c r="R161" t="inlineStr"/>
-      <c r="S161" t="inlineStr"/>
-      <c r="T161" t="inlineStr"/>
       <c r="U161" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14747,13 +14230,9 @@
       <c r="O162" t="n">
         <v>1.1</v>
       </c>
-      <c r="P162" t="inlineStr"/>
       <c r="Q162" t="n">
         <v>0.5</v>
       </c>
-      <c r="R162" t="inlineStr"/>
-      <c r="S162" t="inlineStr"/>
-      <c r="T162" t="inlineStr"/>
       <c r="U162" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14808,7 +14287,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr"/>
       <c r="K163" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -14828,13 +14306,9 @@
       <c r="O163" t="n">
         <v>6.5</v>
       </c>
-      <c r="P163" t="inlineStr"/>
       <c r="Q163" t="n">
         <v>6.6</v>
       </c>
-      <c r="R163" t="inlineStr"/>
-      <c r="S163" t="inlineStr"/>
-      <c r="T163" t="inlineStr"/>
       <c r="U163" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14889,7 +14363,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr"/>
       <c r="K164" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -14909,13 +14382,9 @@
       <c r="O164" t="n">
         <v>5.6</v>
       </c>
-      <c r="P164" t="inlineStr"/>
       <c r="Q164" t="n">
         <v>5.9</v>
       </c>
-      <c r="R164" t="inlineStr"/>
-      <c r="S164" t="inlineStr"/>
-      <c r="T164" t="inlineStr"/>
       <c r="U164" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -14994,13 +14463,9 @@
       <c r="O165" t="n">
         <v>5.9</v>
       </c>
-      <c r="P165" t="inlineStr"/>
       <c r="Q165" t="n">
         <v>6</v>
       </c>
-      <c r="R165" t="inlineStr"/>
-      <c r="S165" t="inlineStr"/>
-      <c r="T165" t="inlineStr"/>
       <c r="U165" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15055,7 +14520,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J166" t="inlineStr"/>
       <c r="K166" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15075,13 +14539,9 @@
       <c r="O166" t="n">
         <v>5.6</v>
       </c>
-      <c r="P166" t="inlineStr"/>
       <c r="Q166" t="n">
         <v>3.1</v>
       </c>
-      <c r="R166" t="inlineStr"/>
-      <c r="S166" t="inlineStr"/>
-      <c r="T166" t="inlineStr"/>
       <c r="U166" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15136,7 +14596,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr"/>
       <c r="K167" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15156,13 +14615,9 @@
       <c r="O167" t="n">
         <v>5.7</v>
       </c>
-      <c r="P167" t="inlineStr"/>
       <c r="Q167" t="n">
         <v>4.8</v>
       </c>
-      <c r="R167" t="inlineStr"/>
-      <c r="S167" t="inlineStr"/>
-      <c r="T167" t="inlineStr"/>
       <c r="U167" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15217,7 +14672,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J168" t="inlineStr"/>
       <c r="K168" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15237,13 +14691,9 @@
       <c r="O168" t="n">
         <v>5.6</v>
       </c>
-      <c r="P168" t="inlineStr"/>
       <c r="Q168" t="n">
         <v>5.6</v>
       </c>
-      <c r="R168" t="inlineStr"/>
-      <c r="S168" t="inlineStr"/>
-      <c r="T168" t="inlineStr"/>
       <c r="U168" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15298,7 +14748,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15318,13 +14767,9 @@
       <c r="O169" t="n">
         <v>5.9</v>
       </c>
-      <c r="P169" t="inlineStr"/>
       <c r="Q169" t="n">
         <v>5.6</v>
       </c>
-      <c r="R169" t="inlineStr"/>
-      <c r="S169" t="inlineStr"/>
-      <c r="T169" t="inlineStr"/>
       <c r="U169" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15379,7 +14824,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr"/>
       <c r="K170" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15393,7 +14837,6 @@
       <c r="M170" t="n">
         <v>33</v>
       </c>
-      <c r="N170" t="inlineStr"/>
       <c r="O170" t="n">
         <v>4.36</v>
       </c>
@@ -15406,8 +14849,6 @@
       <c r="R170" t="n">
         <v>0.58</v>
       </c>
-      <c r="S170" t="inlineStr"/>
-      <c r="T170" t="inlineStr"/>
       <c r="U170" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15462,7 +14903,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr"/>
       <c r="K171" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15476,7 +14916,6 @@
       <c r="M171" t="n">
         <v>33</v>
       </c>
-      <c r="N171" t="inlineStr"/>
       <c r="O171" t="n">
         <v>4.4</v>
       </c>
@@ -15489,8 +14928,6 @@
       <c r="R171" t="n">
         <v>0.6</v>
       </c>
-      <c r="S171" t="inlineStr"/>
-      <c r="T171" t="inlineStr"/>
       <c r="U171" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15545,7 +14982,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J172" t="inlineStr"/>
       <c r="K172" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15559,7 +14995,6 @@
       <c r="M172" t="n">
         <v>33</v>
       </c>
-      <c r="N172" t="inlineStr"/>
       <c r="O172" t="n">
         <v>4.03</v>
       </c>
@@ -15572,8 +15007,6 @@
       <c r="R172" t="n">
         <v>0.498</v>
       </c>
-      <c r="S172" t="inlineStr"/>
-      <c r="T172" t="inlineStr"/>
       <c r="U172" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15628,7 +15061,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J173" t="inlineStr"/>
       <c r="K173" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15642,7 +15074,6 @@
       <c r="M173" t="n">
         <v>33</v>
       </c>
-      <c r="N173" t="inlineStr"/>
       <c r="O173" t="n">
         <v>4.41</v>
       </c>
@@ -15655,8 +15086,6 @@
       <c r="R173" t="n">
         <v>0.593</v>
       </c>
-      <c r="S173" t="inlineStr"/>
-      <c r="T173" t="inlineStr"/>
       <c r="U173" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15701,9 +15130,6 @@
           <t>Ben Degen</t>
         </is>
       </c>
-      <c r="H174" t="inlineStr"/>
-      <c r="I174" t="inlineStr"/>
-      <c r="J174" t="inlineStr"/>
       <c r="K174" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-4o)</t>
@@ -15714,14 +15140,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M174" t="inlineStr"/>
-      <c r="N174" t="inlineStr"/>
-      <c r="O174" t="inlineStr"/>
-      <c r="P174" t="inlineStr"/>
-      <c r="Q174" t="inlineStr"/>
-      <c r="R174" t="inlineStr"/>
-      <c r="S174" t="inlineStr"/>
-      <c r="T174" t="inlineStr"/>
       <c r="U174" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15791,14 +15209,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M175" t="inlineStr"/>
-      <c r="N175" t="inlineStr"/>
-      <c r="O175" t="inlineStr"/>
-      <c r="P175" t="inlineStr"/>
-      <c r="Q175" t="inlineStr"/>
-      <c r="R175" t="inlineStr"/>
-      <c r="S175" t="inlineStr"/>
-      <c r="T175" t="inlineStr"/>
       <c r="U175" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15853,7 +15263,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J176" t="inlineStr"/>
       <c r="K176" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15864,14 +15273,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M176" t="inlineStr"/>
-      <c r="N176" t="inlineStr"/>
-      <c r="O176" t="inlineStr"/>
-      <c r="P176" t="inlineStr"/>
-      <c r="Q176" t="inlineStr"/>
-      <c r="R176" t="inlineStr"/>
-      <c r="S176" t="inlineStr"/>
-      <c r="T176" t="inlineStr"/>
       <c r="U176" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15926,7 +15327,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr"/>
       <c r="K177" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -15937,14 +15337,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M177" t="inlineStr"/>
-      <c r="N177" t="inlineStr"/>
-      <c r="O177" t="inlineStr"/>
-      <c r="P177" t="inlineStr"/>
-      <c r="Q177" t="inlineStr"/>
-      <c r="R177" t="inlineStr"/>
-      <c r="S177" t="inlineStr"/>
-      <c r="T177" t="inlineStr"/>
       <c r="U177" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -15999,7 +15391,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J178" t="inlineStr"/>
       <c r="K178" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -16010,14 +15401,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
-      <c r="O178" t="inlineStr"/>
-      <c r="P178" t="inlineStr"/>
-      <c r="Q178" t="inlineStr"/>
-      <c r="R178" t="inlineStr"/>
-      <c r="S178" t="inlineStr"/>
-      <c r="T178" t="inlineStr"/>
       <c r="U178" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -16201,7 +15584,6 @@
       <c r="S180" t="n">
         <v>1.523</v>
       </c>
-      <c r="T180" t="inlineStr"/>
       <c r="U180" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -16556,12 +15938,6 @@
       <c r="N184" t="n">
         <v>30</v>
       </c>
-      <c r="O184" t="inlineStr"/>
-      <c r="P184" t="inlineStr"/>
-      <c r="Q184" t="inlineStr"/>
-      <c r="R184" t="inlineStr"/>
-      <c r="S184" t="inlineStr"/>
-      <c r="T184" t="inlineStr"/>
       <c r="U184" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -16637,12 +16013,6 @@
       <c r="N185" t="n">
         <v>30</v>
       </c>
-      <c r="O185" t="inlineStr"/>
-      <c r="P185" t="inlineStr"/>
-      <c r="Q185" t="inlineStr"/>
-      <c r="R185" t="inlineStr"/>
-      <c r="S185" t="inlineStr"/>
-      <c r="T185" t="inlineStr"/>
       <c r="U185" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -16718,12 +16088,6 @@
       <c r="N186" t="n">
         <v>30</v>
       </c>
-      <c r="O186" t="inlineStr"/>
-      <c r="P186" t="inlineStr"/>
-      <c r="Q186" t="inlineStr"/>
-      <c r="R186" t="inlineStr"/>
-      <c r="S186" t="inlineStr"/>
-      <c r="T186" t="inlineStr"/>
       <c r="U186" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -16871,7 +16235,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr"/>
       <c r="K188" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -17164,7 +16527,6 @@
       <c r="M191" t="n">
         <v>30</v>
       </c>
-      <c r="N191" t="inlineStr"/>
       <c r="O191" t="n">
         <v>4.47</v>
       </c>
@@ -17177,8 +16539,6 @@
       <c r="R191" t="n">
         <v>1.01</v>
       </c>
-      <c r="S191" t="inlineStr"/>
-      <c r="T191" t="inlineStr"/>
       <c r="U191" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -17251,7 +16611,6 @@
       <c r="M192" t="n">
         <v>30</v>
       </c>
-      <c r="N192" t="inlineStr"/>
       <c r="O192" t="n">
         <v>3.77</v>
       </c>
@@ -17264,8 +16623,6 @@
       <c r="R192" t="n">
         <v>1.06</v>
       </c>
-      <c r="S192" t="inlineStr"/>
-      <c r="T192" t="inlineStr"/>
       <c r="U192" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -17338,7 +16695,6 @@
       <c r="M193" t="n">
         <v>30</v>
       </c>
-      <c r="N193" t="inlineStr"/>
       <c r="O193" t="n">
         <v>1.9</v>
       </c>
@@ -17351,8 +16707,6 @@
       <c r="R193" t="n">
         <v>0.83</v>
       </c>
-      <c r="S193" t="inlineStr"/>
-      <c r="T193" t="inlineStr"/>
       <c r="U193" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -17425,7 +16779,6 @@
       <c r="M194" t="n">
         <v>30</v>
       </c>
-      <c r="N194" t="inlineStr"/>
       <c r="O194" t="n">
         <v>2</v>
       </c>
@@ -17438,8 +16791,6 @@
       <c r="R194" t="n">
         <v>0.82</v>
       </c>
-      <c r="S194" t="inlineStr"/>
-      <c r="T194" t="inlineStr"/>
       <c r="U194" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -17494,7 +16845,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J195" t="inlineStr"/>
       <c r="K195" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -17583,7 +16933,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J196" t="inlineStr"/>
       <c r="K196" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -17672,7 +17021,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J197" t="inlineStr"/>
       <c r="K197" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -17761,7 +17109,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J198" t="inlineStr"/>
       <c r="K198" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -17850,7 +17197,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J199" t="inlineStr"/>
       <c r="K199" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -17939,7 +17285,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr"/>
       <c r="K200" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18028,7 +17373,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J201" t="inlineStr"/>
       <c r="K201" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18045,10 +17389,6 @@
       <c r="N201" t="n">
         <v>75</v>
       </c>
-      <c r="O201" t="inlineStr"/>
-      <c r="P201" t="inlineStr"/>
-      <c r="Q201" t="inlineStr"/>
-      <c r="R201" t="inlineStr"/>
       <c r="S201" t="n">
         <v>0.9065847519076502</v>
       </c>
@@ -18109,7 +17449,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J202" t="inlineStr"/>
       <c r="K202" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18126,10 +17465,6 @@
       <c r="N202" t="n">
         <v>75</v>
       </c>
-      <c r="O202" t="inlineStr"/>
-      <c r="P202" t="inlineStr"/>
-      <c r="Q202" t="inlineStr"/>
-      <c r="R202" t="inlineStr"/>
       <c r="S202" t="n">
         <v>1.481729917096374</v>
       </c>
@@ -18190,7 +17525,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J203" t="inlineStr"/>
       <c r="K203" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18207,10 +17541,6 @@
       <c r="N203" t="n">
         <v>75</v>
       </c>
-      <c r="O203" t="inlineStr"/>
-      <c r="P203" t="inlineStr"/>
-      <c r="Q203" t="inlineStr"/>
-      <c r="R203" t="inlineStr"/>
       <c r="S203" t="n">
         <v>0.3980524448340041</v>
       </c>
@@ -18271,7 +17601,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J204" t="inlineStr"/>
       <c r="K204" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18288,10 +17617,6 @@
       <c r="N204" t="n">
         <v>75</v>
       </c>
-      <c r="O204" t="inlineStr"/>
-      <c r="P204" t="inlineStr"/>
-      <c r="Q204" t="inlineStr"/>
-      <c r="R204" t="inlineStr"/>
       <c r="S204" t="n">
         <v>0.8838388979171358</v>
       </c>
@@ -18352,7 +17677,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J205" t="inlineStr"/>
       <c r="K205" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18369,10 +17693,6 @@
       <c r="N205" t="n">
         <v>75</v>
       </c>
-      <c r="O205" t="inlineStr"/>
-      <c r="P205" t="inlineStr"/>
-      <c r="Q205" t="inlineStr"/>
-      <c r="R205" t="inlineStr"/>
       <c r="S205" t="n">
         <v>1.626328560321788</v>
       </c>
@@ -18433,7 +17753,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J206" t="inlineStr"/>
       <c r="K206" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18450,10 +17769,6 @@
       <c r="N206" t="n">
         <v>75</v>
       </c>
-      <c r="O206" t="inlineStr"/>
-      <c r="P206" t="inlineStr"/>
-      <c r="Q206" t="inlineStr"/>
-      <c r="R206" t="inlineStr"/>
       <c r="S206" t="n">
         <v>0.4841617492266662</v>
       </c>
@@ -18514,7 +17829,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J207" t="inlineStr"/>
       <c r="K207" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18531,10 +17845,6 @@
       <c r="N207" t="n">
         <v>75</v>
       </c>
-      <c r="O207" t="inlineStr"/>
-      <c r="P207" t="inlineStr"/>
-      <c r="Q207" t="inlineStr"/>
-      <c r="R207" t="inlineStr"/>
       <c r="S207" t="n">
         <v>0.9715729061662632</v>
       </c>
@@ -18595,7 +17905,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr"/>
       <c r="K208" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18612,10 +17921,6 @@
       <c r="N208" t="n">
         <v>75</v>
       </c>
-      <c r="O208" t="inlineStr"/>
-      <c r="P208" t="inlineStr"/>
-      <c r="Q208" t="inlineStr"/>
-      <c r="R208" t="inlineStr"/>
       <c r="S208" t="n">
         <v>2.022756301299327</v>
       </c>
@@ -18676,7 +17981,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr"/>
       <c r="K209" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18693,10 +17997,6 @@
       <c r="N209" t="n">
         <v>75</v>
       </c>
-      <c r="O209" t="inlineStr"/>
-      <c r="P209" t="inlineStr"/>
-      <c r="Q209" t="inlineStr"/>
-      <c r="R209" t="inlineStr"/>
       <c r="S209" t="n">
         <v>0.8800437563348654</v>
       </c>
@@ -18757,7 +18057,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J210" t="inlineStr"/>
       <c r="K210" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18774,10 +18073,6 @@
       <c r="N210" t="n">
         <v>75</v>
       </c>
-      <c r="O210" t="inlineStr"/>
-      <c r="P210" t="inlineStr"/>
-      <c r="Q210" t="inlineStr"/>
-      <c r="R210" t="inlineStr"/>
       <c r="S210" t="n">
         <v>0.9300631381640688</v>
       </c>
@@ -18838,7 +18133,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J211" t="inlineStr"/>
       <c r="K211" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -18855,10 +18149,6 @@
       <c r="N211" t="n">
         <v>75</v>
       </c>
-      <c r="O211" t="inlineStr"/>
-      <c r="P211" t="inlineStr"/>
-      <c r="Q211" t="inlineStr"/>
-      <c r="R211" t="inlineStr"/>
       <c r="S211" t="n">
         <v>1.003114844475201</v>
       </c>
@@ -18919,7 +18209,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J212" t="inlineStr"/>
       <c r="K212" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -18936,12 +18225,6 @@
       <c r="N212" t="n">
         <v>118</v>
       </c>
-      <c r="O212" t="inlineStr"/>
-      <c r="P212" t="inlineStr"/>
-      <c r="Q212" t="inlineStr"/>
-      <c r="R212" t="inlineStr"/>
-      <c r="S212" t="inlineStr"/>
-      <c r="T212" t="inlineStr"/>
       <c r="U212" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -18996,7 +18279,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J213" t="inlineStr"/>
       <c r="K213" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19085,7 +18367,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J214" t="inlineStr"/>
       <c r="K214" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19174,7 +18455,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J215" t="inlineStr"/>
       <c r="K215" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19449,7 +18729,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J218" t="inlineStr"/>
       <c r="K218" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19538,7 +18817,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J219" t="inlineStr"/>
       <c r="K219" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19627,7 +18905,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J220" t="inlineStr"/>
       <c r="K220" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19716,7 +18993,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr"/>
       <c r="K221" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19805,7 +19081,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J222" t="inlineStr"/>
       <c r="K222" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19894,7 +19169,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J223" t="inlineStr"/>
       <c r="K223" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -19983,7 +19257,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J224" t="inlineStr"/>
       <c r="K224" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20015,7 +19288,6 @@
       <c r="S224" t="n">
         <v>0.7248</v>
       </c>
-      <c r="T224" t="inlineStr"/>
       <c r="U224" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20070,7 +19342,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J225" t="inlineStr"/>
       <c r="K225" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20087,14 +19358,9 @@
       <c r="N225" t="n">
         <v>54</v>
       </c>
-      <c r="O225" t="inlineStr"/>
-      <c r="P225" t="inlineStr"/>
-      <c r="Q225" t="inlineStr"/>
-      <c r="R225" t="inlineStr"/>
       <c r="S225" t="n">
         <v>0.6752</v>
       </c>
-      <c r="T225" t="inlineStr"/>
       <c r="U225" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20149,7 +19415,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J226" t="inlineStr"/>
       <c r="K226" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20172,8 +19437,6 @@
       <c r="P226" t="n">
         <v>0.65</v>
       </c>
-      <c r="Q226" t="inlineStr"/>
-      <c r="R226" t="inlineStr"/>
       <c r="S226" t="n">
         <v>0.799354543453101</v>
       </c>
@@ -20234,7 +19497,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J227" t="inlineStr"/>
       <c r="K227" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20323,7 +19585,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J228" t="inlineStr"/>
       <c r="K228" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20340,14 +19601,9 @@
       <c r="N228" t="n">
         <v>126</v>
       </c>
-      <c r="O228" t="inlineStr"/>
-      <c r="P228" t="inlineStr"/>
-      <c r="Q228" t="inlineStr"/>
-      <c r="R228" t="inlineStr"/>
       <c r="S228" t="n">
         <v>1.0169</v>
       </c>
-      <c r="T228" t="inlineStr"/>
       <c r="U228" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20402,7 +19658,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J229" t="inlineStr"/>
       <c r="K229" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20419,14 +19674,9 @@
       <c r="N229" t="n">
         <v>121</v>
       </c>
-      <c r="O229" t="inlineStr"/>
-      <c r="P229" t="inlineStr"/>
-      <c r="Q229" t="inlineStr"/>
-      <c r="R229" t="inlineStr"/>
       <c r="S229" t="n">
         <v>0.4685</v>
       </c>
-      <c r="T229" t="inlineStr"/>
       <c r="U229" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20481,7 +19731,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J230" t="inlineStr"/>
       <c r="K230" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20570,7 +19819,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J231" t="inlineStr"/>
       <c r="K231" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -20587,14 +19835,9 @@
       <c r="N231" t="n">
         <v>58</v>
       </c>
-      <c r="O231" t="inlineStr"/>
-      <c r="P231" t="inlineStr"/>
-      <c r="Q231" t="inlineStr"/>
-      <c r="R231" t="inlineStr"/>
       <c r="S231" t="n">
         <v>0.7053</v>
       </c>
-      <c r="T231" t="inlineStr"/>
       <c r="U231" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20649,7 +19892,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -20666,12 +19908,6 @@
       <c r="N232" t="n">
         <v>58</v>
       </c>
-      <c r="O232" t="inlineStr"/>
-      <c r="P232" t="inlineStr"/>
-      <c r="Q232" t="inlineStr"/>
-      <c r="R232" t="inlineStr"/>
-      <c r="S232" t="inlineStr"/>
-      <c r="T232" t="inlineStr"/>
       <c r="U232" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20726,7 +19962,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -20743,12 +19978,6 @@
       <c r="N233" t="n">
         <v>58</v>
       </c>
-      <c r="O233" t="inlineStr"/>
-      <c r="P233" t="inlineStr"/>
-      <c r="Q233" t="inlineStr"/>
-      <c r="R233" t="inlineStr"/>
-      <c r="S233" t="inlineStr"/>
-      <c r="T233" t="inlineStr"/>
       <c r="U233" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20803,7 +20032,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J234" t="inlineStr"/>
       <c r="K234" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -20820,12 +20048,6 @@
       <c r="N234" t="n">
         <v>58</v>
       </c>
-      <c r="O234" t="inlineStr"/>
-      <c r="P234" t="inlineStr"/>
-      <c r="Q234" t="inlineStr"/>
-      <c r="R234" t="inlineStr"/>
-      <c r="S234" t="inlineStr"/>
-      <c r="T234" t="inlineStr"/>
       <c r="U234" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20870,9 +20092,6 @@
           <t>Hartwig H. Hochmair</t>
         </is>
       </c>
-      <c r="H235" t="inlineStr"/>
-      <c r="I235" t="inlineStr"/>
-      <c r="J235" t="inlineStr"/>
       <c r="K235" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -20883,14 +20102,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M235" t="inlineStr"/>
-      <c r="N235" t="inlineStr"/>
-      <c r="O235" t="inlineStr"/>
-      <c r="P235" t="inlineStr"/>
-      <c r="Q235" t="inlineStr"/>
-      <c r="R235" t="inlineStr"/>
-      <c r="S235" t="inlineStr"/>
-      <c r="T235" t="inlineStr"/>
       <c r="U235" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -20972,10 +20183,6 @@
       <c r="P236" t="n">
         <v>0.644</v>
       </c>
-      <c r="Q236" t="inlineStr"/>
-      <c r="R236" t="inlineStr"/>
-      <c r="S236" t="inlineStr"/>
-      <c r="T236" t="inlineStr"/>
       <c r="U236" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21057,10 +20264,6 @@
       <c r="P237" t="n">
         <v>0.635</v>
       </c>
-      <c r="Q237" t="inlineStr"/>
-      <c r="R237" t="inlineStr"/>
-      <c r="S237" t="inlineStr"/>
-      <c r="T237" t="inlineStr"/>
       <c r="U237" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21115,7 +20318,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J238" t="inlineStr"/>
       <c r="K238" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -21138,10 +20340,6 @@
       <c r="P238" t="n">
         <v>0.864</v>
       </c>
-      <c r="Q238" t="inlineStr"/>
-      <c r="R238" t="inlineStr"/>
-      <c r="S238" t="inlineStr"/>
-      <c r="T238" t="inlineStr"/>
       <c r="U238" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21196,7 +20394,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J239" t="inlineStr"/>
       <c r="K239" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -21219,10 +20416,6 @@
       <c r="P239" t="n">
         <v>1.004</v>
       </c>
-      <c r="Q239" t="inlineStr"/>
-      <c r="R239" t="inlineStr"/>
-      <c r="S239" t="inlineStr"/>
-      <c r="T239" t="inlineStr"/>
       <c r="U239" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21298,14 +20491,9 @@
       <c r="N240" t="n">
         <v>100</v>
       </c>
-      <c r="O240" t="inlineStr"/>
-      <c r="P240" t="inlineStr"/>
-      <c r="Q240" t="inlineStr"/>
-      <c r="R240" t="inlineStr"/>
       <c r="S240" t="n">
         <v>0.3815</v>
       </c>
-      <c r="T240" t="inlineStr"/>
       <c r="U240" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21381,14 +20569,9 @@
       <c r="N241" t="n">
         <v>100</v>
       </c>
-      <c r="O241" t="inlineStr"/>
-      <c r="P241" t="inlineStr"/>
-      <c r="Q241" t="inlineStr"/>
-      <c r="R241" t="inlineStr"/>
       <c r="S241" t="n">
         <v>0.4074</v>
       </c>
-      <c r="T241" t="inlineStr"/>
       <c r="U241" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21464,14 +20647,9 @@
       <c r="N242" t="n">
         <v>100</v>
       </c>
-      <c r="O242" t="inlineStr"/>
-      <c r="P242" t="inlineStr"/>
-      <c r="Q242" t="inlineStr"/>
-      <c r="R242" t="inlineStr"/>
       <c r="S242" t="n">
         <v>0.3208</v>
       </c>
-      <c r="T242" t="inlineStr"/>
       <c r="U242" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21547,14 +20725,9 @@
       <c r="N243" t="n">
         <v>100</v>
       </c>
-      <c r="O243" t="inlineStr"/>
-      <c r="P243" t="inlineStr"/>
-      <c r="Q243" t="inlineStr"/>
-      <c r="R243" t="inlineStr"/>
       <c r="S243" t="n">
         <v>0.0767</v>
       </c>
-      <c r="T243" t="inlineStr"/>
       <c r="U243" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21630,14 +20803,9 @@
       <c r="N244" t="n">
         <v>100</v>
       </c>
-      <c r="O244" t="inlineStr"/>
-      <c r="P244" t="inlineStr"/>
-      <c r="Q244" t="inlineStr"/>
-      <c r="R244" t="inlineStr"/>
       <c r="S244" t="n">
         <v>0.4812</v>
       </c>
-      <c r="T244" t="inlineStr"/>
       <c r="U244" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21713,14 +20881,9 @@
       <c r="N245" t="n">
         <v>100</v>
       </c>
-      <c r="O245" t="inlineStr"/>
-      <c r="P245" t="inlineStr"/>
-      <c r="Q245" t="inlineStr"/>
-      <c r="R245" t="inlineStr"/>
       <c r="S245" t="n">
         <v>0.7561</v>
       </c>
-      <c r="T245" t="inlineStr"/>
       <c r="U245" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21796,14 +20959,9 @@
       <c r="N246" t="n">
         <v>100</v>
       </c>
-      <c r="O246" t="inlineStr"/>
-      <c r="P246" t="inlineStr"/>
-      <c r="Q246" t="inlineStr"/>
-      <c r="R246" t="inlineStr"/>
       <c r="S246" t="n">
         <v>0.2451</v>
       </c>
-      <c r="T246" t="inlineStr"/>
       <c r="U246" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21879,14 +21037,9 @@
       <c r="N247" t="n">
         <v>100</v>
       </c>
-      <c r="O247" t="inlineStr"/>
-      <c r="P247" t="inlineStr"/>
-      <c r="Q247" t="inlineStr"/>
-      <c r="R247" t="inlineStr"/>
       <c r="S247" t="n">
         <v>0.2849</v>
       </c>
-      <c r="T247" t="inlineStr"/>
       <c r="U247" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -21962,14 +21115,9 @@
       <c r="N248" t="n">
         <v>100</v>
       </c>
-      <c r="O248" t="inlineStr"/>
-      <c r="P248" t="inlineStr"/>
-      <c r="Q248" t="inlineStr"/>
-      <c r="R248" t="inlineStr"/>
       <c r="S248" t="n">
         <v>0.1664</v>
       </c>
-      <c r="T248" t="inlineStr"/>
       <c r="U248" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -22045,14 +21193,9 @@
       <c r="N249" t="n">
         <v>100</v>
       </c>
-      <c r="O249" t="inlineStr"/>
-      <c r="P249" t="inlineStr"/>
-      <c r="Q249" t="inlineStr"/>
-      <c r="R249" t="inlineStr"/>
       <c r="S249" t="n">
         <v>0.1594</v>
       </c>
-      <c r="T249" t="inlineStr"/>
       <c r="U249" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -22128,14 +21271,9 @@
       <c r="N250" t="n">
         <v>100</v>
       </c>
-      <c r="O250" t="inlineStr"/>
-      <c r="P250" t="inlineStr"/>
-      <c r="Q250" t="inlineStr"/>
-      <c r="R250" t="inlineStr"/>
       <c r="S250" t="n">
         <v>0.3118</v>
       </c>
-      <c r="T250" t="inlineStr"/>
       <c r="U250" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -22211,14 +21349,9 @@
       <c r="N251" t="n">
         <v>100</v>
       </c>
-      <c r="O251" t="inlineStr"/>
-      <c r="P251" t="inlineStr"/>
-      <c r="Q251" t="inlineStr"/>
-      <c r="R251" t="inlineStr"/>
       <c r="S251" t="n">
         <v>0.4612</v>
       </c>
-      <c r="T251" t="inlineStr"/>
       <c r="U251" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -22552,7 +21685,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J255" t="inlineStr"/>
       <c r="K255" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -22641,7 +21773,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -22952,7 +22083,6 @@
       <c r="S259" t="n">
         <v>1.1414</v>
       </c>
-      <c r="T259" t="inlineStr"/>
       <c r="U259" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -23136,7 +22266,6 @@
       <c r="S261" t="n">
         <v>0.8744</v>
       </c>
-      <c r="T261" t="inlineStr"/>
       <c r="U261" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -23227,7 +22356,6 @@
       <c r="S262" t="n">
         <v>1.8202</v>
       </c>
-      <c r="T262" t="inlineStr"/>
       <c r="U262" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -23318,7 +22446,6 @@
       <c r="S263" t="n">
         <v>0.4741</v>
       </c>
-      <c r="T263" t="inlineStr"/>
       <c r="U263" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -23838,7 +22965,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J269" t="inlineStr"/>
       <c r="K269" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -23849,14 +22975,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M269" t="inlineStr"/>
-      <c r="N269" t="inlineStr"/>
-      <c r="O269" t="inlineStr"/>
-      <c r="P269" t="inlineStr"/>
-      <c r="Q269" t="inlineStr"/>
-      <c r="R269" t="inlineStr"/>
-      <c r="S269" t="inlineStr"/>
-      <c r="T269" t="inlineStr"/>
       <c r="U269" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -23926,8 +23044,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M270" t="inlineStr"/>
-      <c r="N270" t="inlineStr"/>
       <c r="O270" t="n">
         <v>6.918</v>
       </c>
@@ -23940,8 +23056,6 @@
       <c r="R270" t="n">
         <v>0.903</v>
       </c>
-      <c r="S270" t="inlineStr"/>
-      <c r="T270" t="inlineStr"/>
       <c r="U270" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -23996,7 +23110,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J271" t="inlineStr"/>
       <c r="K271" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -24085,7 +23198,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr"/>
       <c r="K272" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -24174,7 +23286,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J273" t="inlineStr"/>
       <c r="K273" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -24263,7 +23374,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J274" t="inlineStr"/>
       <c r="K274" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -24352,7 +23462,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr"/>
       <c r="K275" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -24441,7 +23550,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J276" t="inlineStr"/>
       <c r="K276" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -24530,7 +23638,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J277" t="inlineStr"/>
       <c r="K277" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -24619,7 +23726,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr"/>
       <c r="K278" t="inlineStr">
         <is>
           <t>ChatGPT (gpt-3.5-turbo-16k)</t>
@@ -25383,11 +24489,9 @@
       <c r="O286" t="n">
         <v>63.98969</v>
       </c>
-      <c r="P286" t="inlineStr"/>
       <c r="Q286" t="n">
         <v>61.15464</v>
       </c>
-      <c r="R286" t="inlineStr"/>
       <c r="S286" t="n">
         <v>0.2010117055207995</v>
       </c>
@@ -25448,7 +24552,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J287" t="inlineStr"/>
       <c r="K287" t="inlineStr">
         <is>
           <t>GPT-3.5-turbo</t>
@@ -25537,7 +24640,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr"/>
       <c r="K288" t="inlineStr">
         <is>
           <t>GPT-3.5-turbo</t>
@@ -25626,7 +24728,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J289" t="inlineStr"/>
       <c r="K289" t="inlineStr">
         <is>
           <t>GPT-3.5-turbo</t>
@@ -25751,7 +24852,6 @@
       <c r="S290" t="n">
         <v>0.7923</v>
       </c>
-      <c r="T290" t="inlineStr"/>
       <c r="U290" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -25806,7 +24906,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J291" t="inlineStr"/>
       <c r="K291" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -25823,12 +24922,6 @@
       <c r="N291" t="n">
         <v>40</v>
       </c>
-      <c r="O291" t="inlineStr"/>
-      <c r="P291" t="inlineStr"/>
-      <c r="Q291" t="inlineStr"/>
-      <c r="R291" t="inlineStr"/>
-      <c r="S291" t="inlineStr"/>
-      <c r="T291" t="inlineStr"/>
       <c r="U291" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -25883,7 +24976,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J292" t="inlineStr"/>
       <c r="K292" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -25903,13 +24995,9 @@
       <c r="O292" t="n">
         <v>28</v>
       </c>
-      <c r="P292" t="inlineStr"/>
       <c r="Q292" t="n">
         <v>27</v>
       </c>
-      <c r="R292" t="inlineStr"/>
-      <c r="S292" t="inlineStr"/>
-      <c r="T292" t="inlineStr"/>
       <c r="U292" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -25988,13 +25076,9 @@
       <c r="O293" t="n">
         <v>24</v>
       </c>
-      <c r="P293" t="inlineStr"/>
       <c r="Q293" t="n">
         <v>25</v>
       </c>
-      <c r="R293" t="inlineStr"/>
-      <c r="S293" t="inlineStr"/>
-      <c r="T293" t="inlineStr"/>
       <c r="U293" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26049,7 +25133,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J294" t="inlineStr"/>
       <c r="K294" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -26069,13 +25152,9 @@
       <c r="O294" t="n">
         <v>4.2</v>
       </c>
-      <c r="P294" t="inlineStr"/>
       <c r="Q294" t="n">
         <v>3.9</v>
       </c>
-      <c r="R294" t="inlineStr"/>
-      <c r="S294" t="inlineStr"/>
-      <c r="T294" t="inlineStr"/>
       <c r="U294" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26130,7 +25209,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J295" t="inlineStr"/>
       <c r="K295" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -26150,13 +25228,9 @@
       <c r="O295" t="n">
         <v>31</v>
       </c>
-      <c r="P295" t="inlineStr"/>
       <c r="Q295" t="n">
         <v>28</v>
       </c>
-      <c r="R295" t="inlineStr"/>
-      <c r="S295" t="inlineStr"/>
-      <c r="T295" t="inlineStr"/>
       <c r="U295" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26211,7 +25285,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J296" t="inlineStr"/>
       <c r="K296" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -26231,13 +25304,9 @@
       <c r="O296" t="n">
         <v>33.5</v>
       </c>
-      <c r="P296" t="inlineStr"/>
       <c r="Q296" t="n">
         <v>29</v>
       </c>
-      <c r="R296" t="inlineStr"/>
-      <c r="S296" t="inlineStr"/>
-      <c r="T296" t="inlineStr"/>
       <c r="U296" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26292,7 +25361,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J297" t="inlineStr"/>
       <c r="K297" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -26312,13 +25380,9 @@
       <c r="O297" t="n">
         <v>34.4</v>
       </c>
-      <c r="P297" t="inlineStr"/>
       <c r="Q297" t="n">
         <v>28.4</v>
       </c>
-      <c r="R297" t="inlineStr"/>
-      <c r="S297" t="inlineStr"/>
-      <c r="T297" t="inlineStr"/>
       <c r="U297" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26397,13 +25461,9 @@
       <c r="O298" t="n">
         <v>25</v>
       </c>
-      <c r="P298" t="inlineStr"/>
       <c r="Q298" t="n">
         <v>24</v>
       </c>
-      <c r="R298" t="inlineStr"/>
-      <c r="S298" t="inlineStr"/>
-      <c r="T298" t="inlineStr"/>
       <c r="U298" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26482,13 +25542,9 @@
       <c r="O299" t="n">
         <v>33.5</v>
       </c>
-      <c r="P299" t="inlineStr"/>
       <c r="Q299" t="n">
         <v>27</v>
       </c>
-      <c r="R299" t="inlineStr"/>
-      <c r="S299" t="inlineStr"/>
-      <c r="T299" t="inlineStr"/>
       <c r="U299" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26567,13 +25623,9 @@
       <c r="O300" t="n">
         <v>33</v>
       </c>
-      <c r="P300" t="inlineStr"/>
       <c r="Q300" t="n">
         <v>26</v>
       </c>
-      <c r="R300" t="inlineStr"/>
-      <c r="S300" t="inlineStr"/>
-      <c r="T300" t="inlineStr"/>
       <c r="U300" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26628,7 +25680,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J301" t="inlineStr"/>
       <c r="K301" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -26648,13 +25699,9 @@
       <c r="O301" t="n">
         <v>4.65</v>
       </c>
-      <c r="P301" t="inlineStr"/>
       <c r="Q301" t="n">
         <v>4.2</v>
       </c>
-      <c r="R301" t="inlineStr"/>
-      <c r="S301" t="inlineStr"/>
-      <c r="T301" t="inlineStr"/>
       <c r="U301" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -26709,7 +25756,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J302" t="inlineStr"/>
       <c r="K302" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -26729,13 +25775,9 @@
       <c r="O302" t="n">
         <v>5.3</v>
       </c>
-      <c r="P302" t="inlineStr"/>
       <c r="Q302" t="n">
         <v>4.5</v>
       </c>
-      <c r="R302" t="inlineStr"/>
-      <c r="S302" t="inlineStr"/>
-      <c r="T302" t="inlineStr"/>
       <c r="U302" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -27270,18 +26312,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M308" t="inlineStr"/>
-      <c r="N308" t="inlineStr"/>
       <c r="O308" t="n">
         <v>56.40206</v>
       </c>
-      <c r="P308" t="inlineStr"/>
       <c r="Q308" t="n">
         <v>56.68041</v>
       </c>
-      <c r="R308" t="inlineStr"/>
-      <c r="S308" t="inlineStr"/>
-      <c r="T308" t="inlineStr"/>
       <c r="U308" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -27351,18 +26387,12 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M309" t="inlineStr"/>
-      <c r="N309" t="inlineStr"/>
       <c r="O309" t="n">
         <v>63.98969</v>
       </c>
-      <c r="P309" t="inlineStr"/>
       <c r="Q309" t="n">
         <v>61.15464</v>
       </c>
-      <c r="R309" t="inlineStr"/>
-      <c r="S309" t="inlineStr"/>
-      <c r="T309" t="inlineStr"/>
       <c r="U309" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -27432,8 +26462,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M310" t="inlineStr"/>
-      <c r="N310" t="inlineStr"/>
       <c r="O310" t="n">
         <v>7.587629</v>
       </c>
@@ -27446,8 +26474,6 @@
       <c r="R310" t="n">
         <v>7.157</v>
       </c>
-      <c r="S310" t="inlineStr"/>
-      <c r="T310" t="inlineStr"/>
       <c r="U310" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -27502,7 +26528,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J311" t="inlineStr"/>
       <c r="K311" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -27513,8 +26538,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M311" t="inlineStr"/>
-      <c r="N311" t="inlineStr"/>
       <c r="O311" t="n">
         <v>4.556701</v>
       </c>
@@ -27527,8 +26550,6 @@
       <c r="R311" t="n">
         <v>2.761</v>
       </c>
-      <c r="S311" t="inlineStr"/>
-      <c r="T311" t="inlineStr"/>
       <c r="U311" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -27583,7 +26604,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J312" t="inlineStr"/>
       <c r="K312" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -27594,8 +26614,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M312" t="inlineStr"/>
-      <c r="N312" t="inlineStr"/>
       <c r="O312" t="n">
         <v>5.051546</v>
       </c>
@@ -27608,8 +26626,6 @@
       <c r="R312" t="n">
         <v>2.479</v>
       </c>
-      <c r="S312" t="inlineStr"/>
-      <c r="T312" t="inlineStr"/>
       <c r="U312" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -27664,7 +26680,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J313" t="inlineStr"/>
       <c r="K313" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -27675,8 +26690,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M313" t="inlineStr"/>
-      <c r="N313" t="inlineStr"/>
       <c r="O313" t="n">
         <v>4.969072</v>
       </c>
@@ -27689,8 +26702,6 @@
       <c r="R313" t="n">
         <v>2.951</v>
       </c>
-      <c r="S313" t="inlineStr"/>
-      <c r="T313" t="inlineStr"/>
       <c r="U313" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -27730,7 +26741,6 @@
       <c r="F314" t="n">
         <v>2024</v>
       </c>
-      <c r="G314" t="inlineStr"/>
       <c r="H314" t="inlineStr">
         <is>
           <t>Average assignment score</t>
@@ -27777,7 +26787,6 @@
       <c r="S314" t="n">
         <v>1.444</v>
       </c>
-      <c r="T314" t="inlineStr"/>
       <c r="U314" t="inlineStr">
         <is>
           <t>MANUAL_VERIFIED</t>
@@ -27817,7 +26826,6 @@
       <c r="F315" t="n">
         <v>2024</v>
       </c>
-      <c r="G315" t="inlineStr"/>
       <c r="H315" t="inlineStr">
         <is>
           <t>Motivation</t>
@@ -27828,7 +26836,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J315" t="inlineStr"/>
       <c r="K315" t="inlineStr">
         <is>
           <t>GPT-3.5</t>
@@ -27902,7 +26909,6 @@
       <c r="F316" t="n">
         <v>2024</v>
       </c>
-      <c r="G316" t="inlineStr"/>
       <c r="H316" t="inlineStr">
         <is>
           <t>SRL strategy</t>
@@ -27913,7 +26919,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J316" t="inlineStr"/>
       <c r="K316" t="inlineStr">
         <is>
           <t>GPT-3.5</t>
@@ -27987,7 +26992,6 @@
       <c r="F317" t="n">
         <v>2024</v>
       </c>
-      <c r="G317" t="inlineStr"/>
       <c r="H317" t="inlineStr">
         <is>
           <t>Academic performance</t>
@@ -28556,7 +27560,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J323" t="inlineStr"/>
       <c r="K323" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -28645,7 +27648,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J324" t="inlineStr"/>
       <c r="K324" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -28659,13 +27661,6 @@
       <c r="M324" t="n">
         <v>55</v>
       </c>
-      <c r="N324" t="inlineStr"/>
-      <c r="O324" t="inlineStr"/>
-      <c r="P324" t="inlineStr"/>
-      <c r="Q324" t="inlineStr"/>
-      <c r="R324" t="inlineStr"/>
-      <c r="S324" t="inlineStr"/>
-      <c r="T324" t="inlineStr"/>
       <c r="U324" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -28738,13 +27733,6 @@
       <c r="M325" t="n">
         <v>55</v>
       </c>
-      <c r="N325" t="inlineStr"/>
-      <c r="O325" t="inlineStr"/>
-      <c r="P325" t="inlineStr"/>
-      <c r="Q325" t="inlineStr"/>
-      <c r="R325" t="inlineStr"/>
-      <c r="S325" t="inlineStr"/>
-      <c r="T325" t="inlineStr"/>
       <c r="U325" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -28817,13 +27805,6 @@
       <c r="M326" t="n">
         <v>55</v>
       </c>
-      <c r="N326" t="inlineStr"/>
-      <c r="O326" t="inlineStr"/>
-      <c r="P326" t="inlineStr"/>
-      <c r="Q326" t="inlineStr"/>
-      <c r="R326" t="inlineStr"/>
-      <c r="S326" t="inlineStr"/>
-      <c r="T326" t="inlineStr"/>
       <c r="U326" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -28878,7 +27859,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J327" t="inlineStr"/>
       <c r="K327" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -28892,13 +27872,6 @@
       <c r="M327" t="n">
         <v>55</v>
       </c>
-      <c r="N327" t="inlineStr"/>
-      <c r="O327" t="inlineStr"/>
-      <c r="P327" t="inlineStr"/>
-      <c r="Q327" t="inlineStr"/>
-      <c r="R327" t="inlineStr"/>
-      <c r="S327" t="inlineStr"/>
-      <c r="T327" t="inlineStr"/>
       <c r="U327" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -29501,9 +28474,6 @@
           <t>Harsh Kumar; Ruiwei Xiao; Benjamin Lawson; Ilya Musabirov; Jiakai Shi; Xinyuan Wang; Huayin Luo; J. Williams; Anna N. Rafferty; John Stamper; Michael Liut</t>
         </is>
       </c>
-      <c r="H334" t="inlineStr"/>
-      <c r="I334" t="inlineStr"/>
-      <c r="J334" t="inlineStr"/>
       <c r="K334" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -29514,14 +28484,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M334" t="inlineStr"/>
-      <c r="N334" t="inlineStr"/>
-      <c r="O334" t="inlineStr"/>
-      <c r="P334" t="inlineStr"/>
-      <c r="Q334" t="inlineStr"/>
-      <c r="R334" t="inlineStr"/>
-      <c r="S334" t="inlineStr"/>
-      <c r="T334" t="inlineStr"/>
       <c r="U334" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -29566,9 +28528,6 @@
           <t>Lixiang Yan; Roberto Martinez-Maldonado; Yueqiao Jin; Vanessa Echeverria; Mikaela Milesi; Jie Fan; Linxuan Zhao; Riordan Alfredo; Xinyu Li; Dragan Gašević</t>
         </is>
       </c>
-      <c r="H335" t="inlineStr"/>
-      <c r="I335" t="inlineStr"/>
-      <c r="J335" t="inlineStr"/>
       <c r="K335" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -29579,14 +28538,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="M335" t="inlineStr"/>
-      <c r="N335" t="inlineStr"/>
-      <c r="O335" t="inlineStr"/>
-      <c r="P335" t="inlineStr"/>
-      <c r="Q335" t="inlineStr"/>
-      <c r="R335" t="inlineStr"/>
-      <c r="S335" t="inlineStr"/>
-      <c r="T335" t="inlineStr"/>
       <c r="U335" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -29641,7 +28592,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J336" t="inlineStr"/>
       <c r="K336" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -29661,13 +28611,9 @@
       <c r="O336" t="n">
         <v>36.95</v>
       </c>
-      <c r="P336" t="inlineStr"/>
       <c r="Q336" t="n">
         <v>64.44</v>
       </c>
-      <c r="R336" t="inlineStr"/>
-      <c r="S336" t="inlineStr"/>
-      <c r="T336" t="inlineStr"/>
       <c r="U336" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -29746,13 +28692,9 @@
       <c r="O337" t="n">
         <v>35.69</v>
       </c>
-      <c r="P337" t="inlineStr"/>
       <c r="Q337" t="n">
         <v>65.83</v>
       </c>
-      <c r="R337" t="inlineStr"/>
-      <c r="S337" t="inlineStr"/>
-      <c r="T337" t="inlineStr"/>
       <c r="U337" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -29831,13 +28773,9 @@
       <c r="O338" t="n">
         <v>47.09</v>
       </c>
-      <c r="P338" t="inlineStr"/>
       <c r="Q338" t="n">
         <v>53.22</v>
       </c>
-      <c r="R338" t="inlineStr"/>
-      <c r="S338" t="inlineStr"/>
-      <c r="T338" t="inlineStr"/>
       <c r="U338" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -29916,13 +28854,9 @@
       <c r="O339" t="n">
         <v>41.19</v>
       </c>
-      <c r="P339" t="inlineStr"/>
       <c r="Q339" t="n">
         <v>59.74</v>
       </c>
-      <c r="R339" t="inlineStr"/>
-      <c r="S339" t="inlineStr"/>
-      <c r="T339" t="inlineStr"/>
       <c r="U339" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -29977,7 +28911,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J340" t="inlineStr"/>
       <c r="K340" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -29997,13 +28930,9 @@
       <c r="O340" t="n">
         <v>50.58</v>
       </c>
-      <c r="P340" t="inlineStr"/>
       <c r="Q340" t="n">
         <v>49.36</v>
       </c>
-      <c r="R340" t="inlineStr"/>
-      <c r="S340" t="inlineStr"/>
-      <c r="T340" t="inlineStr"/>
       <c r="U340" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30082,13 +29011,9 @@
       <c r="O341" t="n">
         <v>40.85</v>
       </c>
-      <c r="P341" t="inlineStr"/>
       <c r="Q341" t="n">
         <v>60.13</v>
       </c>
-      <c r="R341" t="inlineStr"/>
-      <c r="S341" t="inlineStr"/>
-      <c r="T341" t="inlineStr"/>
       <c r="U341" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30167,13 +29092,9 @@
       <c r="O342" t="n">
         <v>37.42</v>
       </c>
-      <c r="P342" t="inlineStr"/>
       <c r="Q342" t="n">
         <v>63.91</v>
       </c>
-      <c r="R342" t="inlineStr"/>
-      <c r="S342" t="inlineStr"/>
-      <c r="T342" t="inlineStr"/>
       <c r="U342" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30252,13 +29173,9 @@
       <c r="O343" t="n">
         <v>48.06</v>
       </c>
-      <c r="P343" t="inlineStr"/>
       <c r="Q343" t="n">
         <v>52.15</v>
       </c>
-      <c r="R343" t="inlineStr"/>
-      <c r="S343" t="inlineStr"/>
-      <c r="T343" t="inlineStr"/>
       <c r="U343" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30337,13 +29254,9 @@
       <c r="O344" t="n">
         <v>33.42</v>
       </c>
-      <c r="P344" t="inlineStr"/>
       <c r="Q344" t="n">
         <v>68.34</v>
       </c>
-      <c r="R344" t="inlineStr"/>
-      <c r="S344" t="inlineStr"/>
-      <c r="T344" t="inlineStr"/>
       <c r="U344" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30422,13 +29335,9 @@
       <c r="O345" t="n">
         <v>34.78</v>
       </c>
-      <c r="P345" t="inlineStr"/>
       <c r="Q345" t="n">
         <v>66.84</v>
       </c>
-      <c r="R345" t="inlineStr"/>
-      <c r="S345" t="inlineStr"/>
-      <c r="T345" t="inlineStr"/>
       <c r="U345" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30483,7 +29392,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J346" t="inlineStr"/>
       <c r="K346" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -30503,13 +29411,9 @@
       <c r="O346" t="n">
         <v>48.35</v>
       </c>
-      <c r="P346" t="inlineStr"/>
       <c r="Q346" t="n">
         <v>51.83</v>
       </c>
-      <c r="R346" t="inlineStr"/>
-      <c r="S346" t="inlineStr"/>
-      <c r="T346" t="inlineStr"/>
       <c r="U346" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30564,7 +29468,6 @@
           <t>metacognitive</t>
         </is>
       </c>
-      <c r="J347" t="inlineStr"/>
       <c r="K347" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -30584,13 +29487,9 @@
       <c r="O347" t="n">
         <v>39.46</v>
       </c>
-      <c r="P347" t="inlineStr"/>
       <c r="Q347" t="n">
         <v>61.66</v>
       </c>
-      <c r="R347" t="inlineStr"/>
-      <c r="S347" t="inlineStr"/>
-      <c r="T347" t="inlineStr"/>
       <c r="U347" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30630,7 +29529,6 @@
       <c r="F348" t="n">
         <v>2024</v>
       </c>
-      <c r="G348" t="inlineStr"/>
       <c r="H348" t="inlineStr">
         <is>
           <t>Academic Writing Pre-test</t>
@@ -30719,7 +29617,6 @@
       <c r="F349" t="n">
         <v>2024</v>
       </c>
-      <c r="G349" t="inlineStr"/>
       <c r="H349" t="inlineStr">
         <is>
           <t>Academic Writing Post-test</t>
@@ -30813,9 +29710,6 @@
           <t>Alexandre Hudon; Barnabé Kiepura; Myriam Pelletier; Véronique Phan</t>
         </is>
       </c>
-      <c r="H350" t="inlineStr"/>
-      <c r="I350" t="inlineStr"/>
-      <c r="J350" t="inlineStr"/>
       <c r="K350" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -30826,14 +29720,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M350" t="inlineStr"/>
-      <c r="N350" t="inlineStr"/>
-      <c r="O350" t="inlineStr"/>
-      <c r="P350" t="inlineStr"/>
-      <c r="Q350" t="inlineStr"/>
-      <c r="R350" t="inlineStr"/>
-      <c r="S350" t="inlineStr"/>
-      <c r="T350" t="inlineStr"/>
       <c r="U350" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -30873,7 +29759,6 @@
       <c r="F351" t="n">
         <v>2023</v>
       </c>
-      <c r="G351" t="inlineStr"/>
       <c r="H351" t="inlineStr">
         <is>
           <t>knowledge examination</t>
@@ -30977,7 +29862,6 @@
           <t>cognitive</t>
         </is>
       </c>
-      <c r="J352" t="inlineStr"/>
       <c r="K352" t="inlineStr">
         <is>
           <t>not_reported</t>
@@ -31066,7 +29950,6 @@
           <t>behavioral</t>
         </is>
       </c>
-      <c r="J353" t="inlineStr"/>
       <c r="K353" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -31083,12 +29966,6 @@
       <c r="N353" t="n">
         <v>31</v>
       </c>
-      <c r="O353" t="inlineStr"/>
-      <c r="P353" t="inlineStr"/>
-      <c r="Q353" t="inlineStr"/>
-      <c r="R353" t="inlineStr"/>
-      <c r="S353" t="inlineStr"/>
-      <c r="T353" t="inlineStr"/>
       <c r="U353" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31143,7 +30020,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J354" t="inlineStr"/>
       <c r="K354" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -31163,13 +30039,9 @@
       <c r="O354" t="n">
         <v>8.5</v>
       </c>
-      <c r="P354" t="inlineStr"/>
       <c r="Q354" t="n">
         <v>5.7</v>
       </c>
-      <c r="R354" t="inlineStr"/>
-      <c r="S354" t="inlineStr"/>
-      <c r="T354" t="inlineStr"/>
       <c r="U354" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31239,14 +30111,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M355" t="inlineStr"/>
-      <c r="N355" t="inlineStr"/>
-      <c r="O355" t="inlineStr"/>
-      <c r="P355" t="inlineStr"/>
-      <c r="Q355" t="inlineStr"/>
-      <c r="R355" t="inlineStr"/>
-      <c r="S355" t="inlineStr"/>
-      <c r="T355" t="inlineStr"/>
       <c r="U355" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31316,14 +30180,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M356" t="inlineStr"/>
-      <c r="N356" t="inlineStr"/>
-      <c r="O356" t="inlineStr"/>
-      <c r="P356" t="inlineStr"/>
-      <c r="Q356" t="inlineStr"/>
-      <c r="R356" t="inlineStr"/>
-      <c r="S356" t="inlineStr"/>
-      <c r="T356" t="inlineStr"/>
       <c r="U356" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31393,14 +30249,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M357" t="inlineStr"/>
-      <c r="N357" t="inlineStr"/>
-      <c r="O357" t="inlineStr"/>
-      <c r="P357" t="inlineStr"/>
-      <c r="Q357" t="inlineStr"/>
-      <c r="R357" t="inlineStr"/>
-      <c r="S357" t="inlineStr"/>
-      <c r="T357" t="inlineStr"/>
       <c r="U357" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31470,14 +30318,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M358" t="inlineStr"/>
-      <c r="N358" t="inlineStr"/>
-      <c r="O358" t="inlineStr"/>
-      <c r="P358" t="inlineStr"/>
-      <c r="Q358" t="inlineStr"/>
-      <c r="R358" t="inlineStr"/>
-      <c r="S358" t="inlineStr"/>
-      <c r="T358" t="inlineStr"/>
       <c r="U358" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31532,7 +30372,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J359" t="inlineStr"/>
       <c r="K359" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -31543,14 +30382,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="M359" t="inlineStr"/>
-      <c r="N359" t="inlineStr"/>
-      <c r="O359" t="inlineStr"/>
-      <c r="P359" t="inlineStr"/>
-      <c r="Q359" t="inlineStr"/>
-      <c r="R359" t="inlineStr"/>
-      <c r="S359" t="inlineStr"/>
-      <c r="T359" t="inlineStr"/>
       <c r="U359" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31620,18 +30451,12 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M360" t="inlineStr"/>
-      <c r="N360" t="inlineStr"/>
       <c r="O360" t="n">
         <v>29.3</v>
       </c>
       <c r="P360" t="n">
         <v>16.9</v>
       </c>
-      <c r="Q360" t="inlineStr"/>
-      <c r="R360" t="inlineStr"/>
-      <c r="S360" t="inlineStr"/>
-      <c r="T360" t="inlineStr"/>
       <c r="U360" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31701,18 +30526,12 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M361" t="inlineStr"/>
-      <c r="N361" t="inlineStr"/>
       <c r="O361" t="n">
         <v>12.35</v>
       </c>
       <c r="P361" t="n">
         <v>5.33</v>
       </c>
-      <c r="Q361" t="inlineStr"/>
-      <c r="R361" t="inlineStr"/>
-      <c r="S361" t="inlineStr"/>
-      <c r="T361" t="inlineStr"/>
       <c r="U361" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31782,18 +30601,12 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M362" t="inlineStr"/>
-      <c r="N362" t="inlineStr"/>
       <c r="O362" t="n">
         <v>20.37</v>
       </c>
       <c r="P362" t="n">
         <v>20.5</v>
       </c>
-      <c r="Q362" t="inlineStr"/>
-      <c r="R362" t="inlineStr"/>
-      <c r="S362" t="inlineStr"/>
-      <c r="T362" t="inlineStr"/>
       <c r="U362" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31863,18 +30676,12 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M363" t="inlineStr"/>
-      <c r="N363" t="inlineStr"/>
       <c r="O363" t="n">
         <v>10.65</v>
       </c>
       <c r="P363" t="n">
         <v>7.44</v>
       </c>
-      <c r="Q363" t="inlineStr"/>
-      <c r="R363" t="inlineStr"/>
-      <c r="S363" t="inlineStr"/>
-      <c r="T363" t="inlineStr"/>
       <c r="U363" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -31944,18 +30751,12 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M364" t="inlineStr"/>
-      <c r="N364" t="inlineStr"/>
       <c r="O364" t="n">
         <v>6.9</v>
       </c>
       <c r="P364" t="n">
         <v>4.34</v>
       </c>
-      <c r="Q364" t="inlineStr"/>
-      <c r="R364" t="inlineStr"/>
-      <c r="S364" t="inlineStr"/>
-      <c r="T364" t="inlineStr"/>
       <c r="U364" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32025,18 +30826,12 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M365" t="inlineStr"/>
-      <c r="N365" t="inlineStr"/>
       <c r="O365" t="n">
         <v>7.3</v>
       </c>
       <c r="P365" t="n">
         <v>7.82</v>
       </c>
-      <c r="Q365" t="inlineStr"/>
-      <c r="R365" t="inlineStr"/>
-      <c r="S365" t="inlineStr"/>
-      <c r="T365" t="inlineStr"/>
       <c r="U365" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32106,8 +30901,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M366" t="inlineStr"/>
-      <c r="N366" t="inlineStr"/>
       <c r="O366" t="n">
         <v>10.8</v>
       </c>
@@ -32120,8 +30913,6 @@
       <c r="R366" t="n">
         <v>5.59</v>
       </c>
-      <c r="S366" t="inlineStr"/>
-      <c r="T366" t="inlineStr"/>
       <c r="U366" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32191,8 +30982,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M367" t="inlineStr"/>
-      <c r="N367" t="inlineStr"/>
       <c r="O367" t="n">
         <v>7.61</v>
       </c>
@@ -32205,8 +30994,6 @@
       <c r="R367" t="n">
         <v>3.81</v>
       </c>
-      <c r="S367" t="inlineStr"/>
-      <c r="T367" t="inlineStr"/>
       <c r="U367" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32276,8 +31063,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M368" t="inlineStr"/>
-      <c r="N368" t="inlineStr"/>
       <c r="O368" t="n">
         <v>11.42</v>
       </c>
@@ -32287,9 +31072,6 @@
       <c r="Q368" t="n">
         <v>10.2</v>
       </c>
-      <c r="R368" t="inlineStr"/>
-      <c r="S368" t="inlineStr"/>
-      <c r="T368" t="inlineStr"/>
       <c r="U368" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32359,8 +31141,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M369" t="inlineStr"/>
-      <c r="N369" t="inlineStr"/>
       <c r="O369" t="n">
         <v>9.869999999999999</v>
       </c>
@@ -32373,8 +31153,6 @@
       <c r="R369" t="n">
         <v>5.09</v>
       </c>
-      <c r="S369" t="inlineStr"/>
-      <c r="T369" t="inlineStr"/>
       <c r="U369" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32444,8 +31222,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M370" t="inlineStr"/>
-      <c r="N370" t="inlineStr"/>
       <c r="O370" t="n">
         <v>6.95</v>
       </c>
@@ -32458,8 +31234,6 @@
       <c r="R370" t="n">
         <v>3.97</v>
       </c>
-      <c r="S370" t="inlineStr"/>
-      <c r="T370" t="inlineStr"/>
       <c r="U370" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32529,8 +31303,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M371" t="inlineStr"/>
-      <c r="N371" t="inlineStr"/>
       <c r="O371" t="n">
         <v>9.84</v>
       </c>
@@ -32540,9 +31312,6 @@
       <c r="Q371" t="n">
         <v>7.47</v>
       </c>
-      <c r="R371" t="inlineStr"/>
-      <c r="S371" t="inlineStr"/>
-      <c r="T371" t="inlineStr"/>
       <c r="U371" t="inlineStr">
         <is>
           <t>OCR_VERIFIED</t>
@@ -32582,10 +31351,6 @@
       <c r="F372" t="n">
         <v>2018</v>
       </c>
-      <c r="G372" t="inlineStr"/>
-      <c r="H372" t="inlineStr"/>
-      <c r="I372" t="inlineStr"/>
-      <c r="J372" t="inlineStr"/>
       <c r="K372" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -32596,14 +31361,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="M372" t="inlineStr"/>
-      <c r="N372" t="inlineStr"/>
-      <c r="O372" t="inlineStr"/>
-      <c r="P372" t="inlineStr"/>
-      <c r="Q372" t="inlineStr"/>
-      <c r="R372" t="inlineStr"/>
-      <c r="S372" t="inlineStr"/>
-      <c r="T372" t="inlineStr"/>
       <c r="U372" t="inlineStr">
         <is>
           <t>NOT_CHECKED</t>
@@ -32640,8 +31397,6 @@
           <t>The Effect of Flipped Interactive Learning (FIL) Based on ChatGPT on Students’ Skills in a Large Programming Class</t>
         </is>
       </c>
-      <c r="F373" t="inlineStr"/>
-      <c r="G373" t="inlineStr"/>
       <c r="H373" t="inlineStr">
         <is>
           <t>programming skills</t>
@@ -32750,8 +31505,6 @@
           <t>apply</t>
         </is>
       </c>
-      <c r="K374" t="inlineStr"/>
-      <c r="L374" t="inlineStr"/>
       <c r="M374" t="n">
         <v>21</v>
       </c>
@@ -32830,9 +31583,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J375" t="inlineStr"/>
-      <c r="K375" t="inlineStr"/>
-      <c r="L375" t="inlineStr"/>
       <c r="M375" t="n">
         <v>21</v>
       </c>
@@ -32911,9 +31661,6 @@
           <t>affective</t>
         </is>
       </c>
-      <c r="J376" t="inlineStr"/>
-      <c r="K376" t="inlineStr"/>
-      <c r="L376" t="inlineStr"/>
       <c r="M376" t="n">
         <v>21</v>
       </c>
@@ -33108,7 +31855,6 @@
       <c r="C4" t="n">
         <v>2025</v>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -33279,7 +32025,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
         <v>1</v>
       </c>
@@ -33382,7 +32127,6 @@
       <c r="C11" t="n">
         <v>2025</v>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -33793,7 +32537,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="n">
         <v>11</v>
       </c>
@@ -33871,7 +32614,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="n">
         <v>12</v>
       </c>
@@ -33934,7 +32676,6 @@
       <c r="C25" t="n">
         <v>2025</v>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -34065,7 +32806,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="n">
         <v>1</v>
       </c>
@@ -34423,7 +33163,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="n">
         <v>1</v>
       </c>
@@ -34661,7 +33400,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="n">
         <v>1</v>
       </c>
@@ -34939,7 +33677,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="n">
         <v>6</v>
       </c>
@@ -34962,7 +33699,6 @@
       <c r="C51" t="n">
         <v>2024</v>
       </c>
-      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>GPT-3.5</t>
@@ -35133,7 +33869,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
       <c r="H55" t="n">
         <v>1</v>
       </c>
@@ -35171,7 +33906,6 @@
           <t>RCT</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
       <c r="H56" t="n">
         <v>1</v>
       </c>
@@ -35234,7 +33968,6 @@
       <c r="C58" t="n">
         <v>2024</v>
       </c>
-      <c r="D58" t="inlineStr"/>
       <c r="E58" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -35285,7 +34018,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
       <c r="H59" t="n">
         <v>1</v>
       </c>
@@ -35308,7 +34040,6 @@
       <c r="C60" t="n">
         <v>2023</v>
       </c>
-      <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -35439,7 +34170,6 @@
           <t>not_reported</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
       <c r="H63" t="n">
         <v>5</v>
       </c>
@@ -35477,7 +34207,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
       <c r="H64" t="n">
         <v>12</v>
       </c>
@@ -35500,7 +34229,6 @@
       <c r="C65" t="n">
         <v>2018</v>
       </c>
-      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -35511,7 +34239,6 @@
           <t>quasi-experimental</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
       <c r="H65" t="n">
         <v>1</v>
       </c>
@@ -35531,8 +34258,6 @@
           <t>The Effect of Flipped Interactive Learning (FIL) Based on ChatGPT on Students’ Skills in a Large Programming Class</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
           <t>ChatGPT</t>
@@ -35573,8 +34298,6 @@
           <t>Ramazan Yilmaz; Fatma Gizem Karaoglan Yilmaz</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="n">
         <v>21</v>
       </c>
@@ -35878,4 +34601,137 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Study_ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Exclusion_Reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Rommel et al.</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Development of adaptive and emotionally responsive tutoring</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>No quantitative learning outcome data</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Satoru et al.</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Generative AI and CEFR Levels Evaluating</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Assessment tool validation, not intervention study</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jenny et al.</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Using Generative AI to Promote Psychological topic</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Qualitative/descriptive study, no effect sizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>61</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Pablo et al.</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Thinking Critically about Scientific Information</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>No control group comparison</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>